<commit_message>
Excluding water years now works for public users
</commit_message>
<xml_diff>
--- a/Demand/InputData/Watershed_Demand_Dataset_Paths.xlsx
+++ b/Demand/InputData/Watershed_Demand_Dataset_Paths.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cawaterboards.sharepoint.com/DWR/SDA/Shared Documents/Program Watersheds/4. Demand Data Tracking/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aprashar\Documents\Github\DWRAT_DataScraping\Demand\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1049" documentId="13_ncr:1_{E64811C1-A6C0-44B2-A03A-F7D16B36D838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EA56634-4979-4C64-A7FE-3FF38D48BBFA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0730F106-7ADB-4B44-AC33-8DA3E84392C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8961FACC-9C35-4F39-BB8E-E3D4A8B78A2C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8961FACC-9C35-4F39-BB8E-E3D4A8B78A2C}"/>
   </bookViews>
   <sheets>
     <sheet name="Main_Sheet" sheetId="1" r:id="rId1"/>
@@ -121,7 +121,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="338">
   <si>
     <t>Info</t>
   </si>
@@ -1184,6 +1184,21 @@
   </si>
   <si>
     <t>C:\Users\amoussalli\Downloads\Mattole_HUC8\HUC8</t>
+  </si>
+  <si>
+    <t>Delta</t>
+  </si>
+  <si>
+    <t>DL</t>
+  </si>
+  <si>
+    <t>C:\Users\aprashar\Documents\Github\DWRAT_DataScraping\Demand\InputData\i03_LegalDeltaBoundary.geojson</t>
+  </si>
+  <si>
+    <t>EXCLUDED_REPORTING_YEARS</t>
+  </si>
+  <si>
+    <t>2021;2022</t>
   </si>
 </sst>
 </file>
@@ -1424,7 +1439,19 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="23">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thick">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1578,33 +1605,30 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C711BD3A-4AB6-4D67-BD42-3FB9626AC287}" name="Table2" displayName="Table2" ref="A2:AW15" totalsRowShown="0" headerRowDxfId="21">
-  <autoFilter ref="A2:AW15" xr:uid="{C711BD3A-4AB6-4D67-BD42-3FB9626AC287}"/>
-  <tableColumns count="49">
-    <tableColumn id="1" xr3:uid="{776E81EE-3D82-4F84-A7E1-E5AFAD450426}" name="INDEX" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C711BD3A-4AB6-4D67-BD42-3FB9626AC287}" name="Table2" displayName="Table2" ref="A2:AX16" totalsRowShown="0" headerRowDxfId="22">
+  <autoFilter ref="A2:AX16" xr:uid="{C711BD3A-4AB6-4D67-BD42-3FB9626AC287}"/>
+  <tableColumns count="50">
+    <tableColumn id="1" xr3:uid="{776E81EE-3D82-4F84-A7E1-E5AFAD450426}" name="INDEX" dataDxfId="21">
       <calculatedColumnFormula>ROW(B3) - 2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{D398884F-42D5-47C1-B3FC-B226E40F56C9}" name="NAME"/>
-    <tableColumn id="3" xr3:uid="{4FACAB44-BBA1-4B8A-BF3E-060B26921A3E}" name="ID" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{321EF454-3BDA-4FED-84A0-242C6CFD30CE}" name="WATERSHED_BOUNDARY_DATABASE_PATH" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{18A10455-06B2-4B6E-9D24-48D247873D5B}" name="WATERSHED_BOUNDARY_LAYER_NAME" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{A44DDF5D-002A-45F2-87CD-E4BDCC91F051}" name="IS_SHAREPOINT_PATH_WATERSHED_BOUNDARY" dataDxfId="16"/>
-    <tableColumn id="26" xr3:uid="{A34CFBB5-3CA3-471B-8C9D-FFD2620BEE67}" name="WATERSHED_COLUMN_SEARCH_STRING" dataDxfId="15"/>
-    <tableColumn id="27" xr3:uid="{B752EE02-609B-45A5-9A8B-B23ECE55E9DF}" name="SOURCE_NAME_COLUMN_SEARCH_STRING" dataDxfId="14"/>
-    <tableColumn id="28" xr3:uid="{6784E5FE-7D00-4755-B3D1-7E214D9D6EFA}" name="TRIB_DESC_COLUMN_SEARCH_STRING" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{1AF87C52-D944-4D7B-A074-D3ED32FFAA03}" name="WATERSHED_EXIT_POINT_INDEX" dataDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{AC0EB44C-3D57-4B3D-B2AA-2B91C7692534}" name="GIS_PREPROCESSING_SPREADSHEET_PATH" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{4FACAB44-BBA1-4B8A-BF3E-060B26921A3E}" name="ID" dataDxfId="20"/>
+    <tableColumn id="51" xr3:uid="{B7595ECA-A15A-4155-8B15-4800F18CCDFD}" name="EXCLUDED_REPORTING_YEARS" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{321EF454-3BDA-4FED-84A0-242C6CFD30CE}" name="WATERSHED_BOUNDARY_DATABASE_PATH" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{18A10455-06B2-4B6E-9D24-48D247873D5B}" name="WATERSHED_BOUNDARY_LAYER_NAME" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{A44DDF5D-002A-45F2-87CD-E4BDCC91F051}" name="IS_SHAREPOINT_PATH_WATERSHED_BOUNDARY" dataDxfId="17"/>
+    <tableColumn id="26" xr3:uid="{A34CFBB5-3CA3-471B-8C9D-FFD2620BEE67}" name="WATERSHED_COLUMN_SEARCH_STRING" dataDxfId="16"/>
+    <tableColumn id="27" xr3:uid="{B752EE02-609B-45A5-9A8B-B23ECE55E9DF}" name="SOURCE_NAME_COLUMN_SEARCH_STRING" dataDxfId="15"/>
+    <tableColumn id="28" xr3:uid="{6784E5FE-7D00-4755-B3D1-7E214D9D6EFA}" name="TRIB_DESC_COLUMN_SEARCH_STRING" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{1AF87C52-D944-4D7B-A074-D3ED32FFAA03}" name="WATERSHED_EXIT_POINT_INDEX" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{AC0EB44C-3D57-4B3D-B2AA-2B91C7692534}" name="GIS_PREPROCESSING_SPREADSHEET_PATH" dataDxfId="12"/>
     <tableColumn id="9" xr3:uid="{B00750ED-07CA-4479-AFF3-3151E1E0F833}" name="GIS_PREPROCESSING_WORKSHEET_NAME"/>
-    <tableColumn id="10" xr3:uid="{812E332A-6EEB-4CA3-A2D6-4547CD7C54A4}" name="IS_SHAREPOINT_PATH_GIS_PREPROCESSING_SPREADSHEET" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{812E332A-6EEB-4CA3-A2D6-4547CD7C54A4}" name="IS_SHAREPOINT_PATH_GIS_PREPROCESSING_SPREADSHEET" dataDxfId="11"/>
     <tableColumn id="46" xr3:uid="{49AF8B55-F40C-42E4-A524-B49C4F8CF00A}" name="EWRIMS_REPORTS_FOLDER_PATH"/>
     <tableColumn id="29" xr3:uid="{D03F612F-DD50-4A34-9AC0-CD6674450BE6}" name="POD_APPLICATION_NUMBER_SPREADSHEET_PATH"/>
     <tableColumn id="30" xr3:uid="{C2AD24F7-0584-49C9-A672-C8DD7146A417}" name="POD_APPLICATION_NUMBER_WORKSHEET_NAME"/>
-    <tableColumn id="31" xr3:uid="{66CE7497-E596-413F-8921-544BB74C3DD7}" name="IS_SHAREPOINT_PATH_POD_APPLICATION_NUMBER_SPREADSHEET" dataDxfId="9"/>
+    <tableColumn id="31" xr3:uid="{66CE7497-E596-413F-8921-544BB74C3DD7}" name="IS_SHAREPOINT_PATH_POD_APPLICATION_NUMBER_SPREADSHEET" dataDxfId="10"/>
     <tableColumn id="11" xr3:uid="{5DB7ED87-871F-4C06-8BF4-35668661F916}" name="QAQC_UNIT_CONVERSION_ERRORS_SPREADSHEET_PATH"/>
     <tableColumn id="12" xr3:uid="{3442F1AA-5583-49F9-916A-1D3BE29BF0E0}" name="QAQC_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME"/>
     <tableColumn id="13" xr3:uid="{DCBCDD9C-561B-45B9-A277-8DC826228F9D}" name="IS_SHAREPOINT_PATH_QAQC_UNIT_CONVERSION_ERRORS_SPREADSHEET"/>
@@ -1612,21 +1636,21 @@
     <tableColumn id="24" xr3:uid="{4402E847-8344-4AC0-83BD-027C2C85F955}" name="QAQC_MEASUREMENT_VALUES_SPREADSHEET_WORKSHEET_NAME"/>
     <tableColumn id="23" xr3:uid="{BF3DBB2A-B4D9-497B-9AA9-202689EB04F8}" name="IS_SHAREPOINT_PATH_QAQC_MEASUREMENT_VALUES"/>
     <tableColumn id="14" xr3:uid="{1F6934E6-F4A1-4438-909C-60C56721DB48}" name="QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET_PATH"/>
-    <tableColumn id="15" xr3:uid="{B0C47A36-9A34-4BBF-8403-827FA51FD727}" name="QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME" dataDxfId="8"/>
-    <tableColumn id="16" xr3:uid="{538377CD-C686-44C6-87ED-6ABD5DF88F83}" name="IS_SHAREPOINT_PATH_QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET" dataDxfId="7"/>
-    <tableColumn id="17" xr3:uid="{C9FB89DE-1AD6-4FEC-8961-82B10F599F29}" name="QAQC_DUPLICATE_REPORTING_SPREADSHEET_PATH" dataDxfId="6"/>
-    <tableColumn id="18" xr3:uid="{0E0BCAD4-6245-49D8-AE35-419FAD1FA06B}" name="QAQC_DUPLICATE_REPORTING_WORKSHEET_NAME" dataDxfId="5"/>
-    <tableColumn id="19" xr3:uid="{5AF9174D-850A-401C-8553-F941816CB39D}" name="IS_SHAREPOINT_PATH_QAQC_DUPLICATE_REPORTING_SPREADSHEET" dataDxfId="4"/>
+    <tableColumn id="15" xr3:uid="{B0C47A36-9A34-4BBF-8403-827FA51FD727}" name="QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME" dataDxfId="9"/>
+    <tableColumn id="16" xr3:uid="{538377CD-C686-44C6-87ED-6ABD5DF88F83}" name="IS_SHAREPOINT_PATH_QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET" dataDxfId="8"/>
+    <tableColumn id="17" xr3:uid="{C9FB89DE-1AD6-4FEC-8961-82B10F599F29}" name="QAQC_DUPLICATE_REPORTING_SPREADSHEET_PATH" dataDxfId="7"/>
+    <tableColumn id="18" xr3:uid="{0E0BCAD4-6245-49D8-AE35-419FAD1FA06B}" name="QAQC_DUPLICATE_REPORTING_WORKSHEET_NAME" dataDxfId="6"/>
+    <tableColumn id="19" xr3:uid="{5AF9174D-850A-401C-8553-F941816CB39D}" name="IS_SHAREPOINT_PATH_QAQC_DUPLICATE_REPORTING_SPREADSHEET" dataDxfId="5"/>
     <tableColumn id="42" xr3:uid="{2E400177-88F2-41C0-8BDB-5818D102917B}" name="NA_REPORTS_SPREADSHEET_PATH"/>
     <tableColumn id="41" xr3:uid="{3CD8CF08-7BC6-467E-8C6D-253F1DFF6541}" name="NA_REPORTS_WORKSHEET_NAME"/>
-    <tableColumn id="40" xr3:uid="{8AC94F1A-65B4-4A42-AA0D-212073E77362}" name="IS_SHAREPOINT_PATH_NA_REPORTS_SPREADSHEET" dataDxfId="3"/>
+    <tableColumn id="40" xr3:uid="{8AC94F1A-65B4-4A42-AA0D-212073E77362}" name="IS_SHAREPOINT_PATH_NA_REPORTS_SPREADSHEET" dataDxfId="4"/>
     <tableColumn id="32" xr3:uid="{281E90F9-0915-4C7E-B4B0-D3A865435D1A}" name="POD_COORDINATES_SPREADSHEET_PATH"/>
     <tableColumn id="33" xr3:uid="{11DF8B48-852D-46FB-8541-B4DBAB7A1AB6}" name="POD_COORDINATES_WORKSHEET_NAME"/>
     <tableColumn id="35" xr3:uid="{FE79FDB1-2CE3-42C6-90E4-3857101E5E8A}" name="IS_SHAREPOINT_PATH_POD_COORDINATES_SPREADSHEET"/>
     <tableColumn id="34" xr3:uid="{47BF0670-01C9-478D-9F45-481314955B4E}" name="POD_COORDINATES_REFERENCE_SYSTEM"/>
     <tableColumn id="20" xr3:uid="{6557FF05-7172-4057-9259-C83EA504646F}" name="SUBBASIN_POLYGONS_DATABASE_PATH"/>
     <tableColumn id="21" xr3:uid="{71DF2163-A7B7-471B-909E-7C0B1372B75B}" name="SUBBASIN_POLYGONS_LAYER_NAME"/>
-    <tableColumn id="22" xr3:uid="{4731AD94-4A54-4E5D-8226-C553D6203196}" name="IS_SHAREPOINT_PATH_SUBBASIN_POLYGONS" dataDxfId="2"/>
+    <tableColumn id="22" xr3:uid="{4731AD94-4A54-4E5D-8226-C553D6203196}" name="IS_SHAREPOINT_PATH_SUBBASIN_POLYGONS" dataDxfId="3"/>
     <tableColumn id="36" xr3:uid="{79EB03EB-27F7-40E3-B85F-9A85C71A18D9}" name="SUBBASIN_FIELD_ID_NAMES"/>
     <tableColumn id="45" xr3:uid="{1FF3574F-AF8C-465E-B27F-34F613EB9725}" name="CONNECTIVITY_MATRIX_SPREADSHEET_PATH"/>
     <tableColumn id="44" xr3:uid="{F6CF9B50-BFEF-4799-8DBA-489BED7B2892}" name="CONNECTIVITY_MATRIX_WORKSHEET_NAME"/>
@@ -1646,9 +1670,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{14D3AF92-57CC-48E0-916C-527CCD353E2B}" name="Table4" displayName="Table4" ref="A1:C47" totalsRowShown="0">
   <autoFilter ref="A1:C47" xr:uid="{14D3AF92-57CC-48E0-916C-527CCD353E2B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{47B19E1B-043A-4C10-A456-3179E3432197}" name="COLUMN_NAME" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{47B19E1B-043A-4C10-A456-3179E3432197}" name="COLUMN_NAME" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{7C95D3E6-5AC8-446C-AA32-9C6FCCE24F43}" name="DEFINITION"/>
-    <tableColumn id="3" xr3:uid="{4D580C7B-D92C-44C5-BD46-100E46839D1B}" name="DESCRIPTION" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{4D580C7B-D92C-44C5-BD46-100E46839D1B}" name="DESCRIPTION" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1971,67 +1995,68 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24A2F77B-58D1-4171-AA16-A7B2F203ADC2}">
-  <dimension ref="A1:AW15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AX16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.5703125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="58" style="12" customWidth="1"/>
-    <col min="6" max="6" width="45.42578125" style="12" customWidth="1"/>
-    <col min="7" max="7" width="40" style="12" customWidth="1"/>
-    <col min="8" max="8" width="58" style="12" customWidth="1"/>
-    <col min="9" max="9" width="58" style="2" customWidth="1"/>
-    <col min="10" max="10" width="58" style="15" customWidth="1"/>
-    <col min="11" max="11" width="58" style="2" customWidth="1"/>
-    <col min="12" max="12" width="52" customWidth="1"/>
-    <col min="13" max="13" width="57" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="60.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="91.5703125" customWidth="1"/>
-    <col min="16" max="16" width="52" customWidth="1"/>
-    <col min="17" max="17" width="63.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="90.5703125" customWidth="1"/>
-    <col min="19" max="19" width="53.42578125" customWidth="1"/>
-    <col min="20" max="20" width="70" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="136.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="63.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="57.42578125" customWidth="1"/>
-    <col min="24" max="24" width="112.42578125" customWidth="1"/>
-    <col min="25" max="25" width="48.5703125" style="2" customWidth="1"/>
-    <col min="26" max="26" width="85.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="51.5703125" style="2" customWidth="1"/>
-    <col min="28" max="28" width="48.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="65.5703125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="94.5703125" customWidth="1"/>
-    <col min="31" max="32" width="65.5703125" customWidth="1"/>
-    <col min="33" max="33" width="65" customWidth="1"/>
-    <col min="34" max="36" width="65.5703125" customWidth="1"/>
-    <col min="37" max="37" width="43.42578125" customWidth="1"/>
-    <col min="38" max="38" width="39.42578125" customWidth="1"/>
-    <col min="39" max="39" width="46.5703125" customWidth="1"/>
-    <col min="40" max="40" width="37.42578125" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="39.42578125" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="38.42578125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="53.5703125" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="52.42578125" hidden="1" customWidth="1"/>
-    <col min="45" max="45" width="47.5703125" hidden="1" customWidth="1"/>
-    <col min="46" max="46" width="49.5703125" hidden="1" customWidth="1"/>
-    <col min="47" max="47" width="62.42578125" customWidth="1"/>
-    <col min="48" max="48" width="42.5703125" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="59.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" customWidth="1"/>
+    <col min="5" max="5" width="61.5546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="58" style="12" customWidth="1"/>
+    <col min="7" max="7" width="45.44140625" style="12" customWidth="1"/>
+    <col min="8" max="8" width="40" style="12" customWidth="1"/>
+    <col min="9" max="9" width="58" style="12" customWidth="1"/>
+    <col min="10" max="10" width="58" style="2" customWidth="1"/>
+    <col min="11" max="11" width="58" style="15" customWidth="1"/>
+    <col min="12" max="12" width="58" style="2" customWidth="1"/>
+    <col min="13" max="13" width="52" customWidth="1"/>
+    <col min="14" max="14" width="57" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="60.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="91.5546875" customWidth="1"/>
+    <col min="17" max="17" width="52" customWidth="1"/>
+    <col min="18" max="18" width="63.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="90.5546875" customWidth="1"/>
+    <col min="20" max="20" width="53.44140625" customWidth="1"/>
+    <col min="21" max="21" width="70" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="136.5546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="63.44140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="57.44140625" customWidth="1"/>
+    <col min="25" max="25" width="112.44140625" customWidth="1"/>
+    <col min="26" max="26" width="48.5546875" style="2" customWidth="1"/>
+    <col min="27" max="27" width="85.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="51.5546875" style="2" customWidth="1"/>
+    <col min="29" max="29" width="48.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="65.5546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="94.5546875" customWidth="1"/>
+    <col min="32" max="33" width="65.5546875" customWidth="1"/>
+    <col min="34" max="34" width="65" customWidth="1"/>
+    <col min="35" max="37" width="65.5546875" customWidth="1"/>
+    <col min="38" max="38" width="43.44140625" customWidth="1"/>
+    <col min="39" max="39" width="39.44140625" customWidth="1"/>
+    <col min="40" max="40" width="46.5546875" customWidth="1"/>
+    <col min="41" max="41" width="37.44140625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="39.44140625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="38.44140625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="53.5546875" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="52.44140625" hidden="1" customWidth="1"/>
+    <col min="46" max="46" width="47.5546875" hidden="1" customWidth="1"/>
+    <col min="47" max="47" width="49.5546875" hidden="1" customWidth="1"/>
+    <col min="48" max="48" width="62.44140625" customWidth="1"/>
+    <col min="49" max="49" width="42.5546875" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="59.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="28"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="26"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="25" t="s">
+        <v>1</v>
+      </c>
       <c r="F1" s="26"/>
       <c r="G1" s="26"/>
       <c r="H1" s="26"/>
@@ -2039,17 +2064,17 @@
       <c r="J1" s="26"/>
       <c r="K1" s="26"/>
       <c r="L1" s="26"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="33" t="s">
+      <c r="M1" s="26"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="34"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="30" t="s">
+      <c r="Q1" s="34"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="S1" s="31"/>
       <c r="T1" s="31"/>
       <c r="U1" s="31"/>
       <c r="V1" s="31"/>
@@ -2059,16 +2084,16 @@
       <c r="Z1" s="31"/>
       <c r="AA1" s="31"/>
       <c r="AB1" s="31"/>
-      <c r="AC1" s="32"/>
-      <c r="AD1" s="36" t="s">
+      <c r="AC1" s="31"/>
+      <c r="AD1" s="32"/>
+      <c r="AE1" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="AE1" s="37"/>
-      <c r="AF1" s="38"/>
-      <c r="AG1" s="23" t="s">
+      <c r="AF1" s="37"/>
+      <c r="AG1" s="38"/>
+      <c r="AH1" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="AH1" s="24"/>
       <c r="AI1" s="24"/>
       <c r="AJ1" s="24"/>
       <c r="AK1" s="24"/>
@@ -2084,8 +2109,9 @@
       <c r="AU1" s="24"/>
       <c r="AV1" s="24"/>
       <c r="AW1" s="24"/>
-    </row>
-    <row r="2" spans="1:49" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AX1" s="24"/>
+    </row>
+    <row r="2" spans="1:50" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
@@ -2095,146 +2121,149 @@
       <c r="C2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="E2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="F2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="G2" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="H2" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="I2" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="J2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="J2" s="19" t="s">
+      <c r="K2" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="L2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="N2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="O2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="P2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="Q2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="R2" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="S2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="W2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="X2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="Y2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="Y2" s="13" t="s">
+      <c r="Z2" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="Z2" s="13" t="s">
+      <c r="AA2" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="AA2" s="13" t="s">
+      <c r="AB2" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="AB2" s="13" t="s">
+      <c r="AC2" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="AC2" s="5" t="s">
+      <c r="AD2" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="AD2" s="8" t="s">
+      <c r="AE2" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="AE2" s="8" t="s">
+      <c r="AF2" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="AF2" s="16" t="s">
+      <c r="AG2" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="AG2" s="8" t="s">
+      <c r="AH2" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="AH2" s="8" t="s">
+      <c r="AI2" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="AI2" s="8" t="s">
+      <c r="AJ2" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="AJ2" s="8" t="s">
+      <c r="AK2" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="AK2" s="4" t="s">
+      <c r="AL2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="AL2" s="4" t="s">
+      <c r="AM2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="AM2" s="4" t="s">
+      <c r="AN2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="AN2" s="4" t="s">
+      <c r="AO2" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="AO2" s="4" t="s">
+      <c r="AP2" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="AP2" s="4" t="s">
+      <c r="AQ2" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="AQ2" s="4" t="s">
+      <c r="AR2" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="AR2" s="4" t="s">
+      <c r="AS2" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="AS2" s="4" t="s">
+      <c r="AT2" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="AT2" s="4" t="s">
+      <c r="AU2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="AU2" s="18" t="s">
+      <c r="AV2" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="AV2" s="18" t="s">
+      <c r="AW2" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="AW2" s="18" t="s">
+      <c r="AX2" s="18" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:49" s="11" customFormat="1" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:50" s="11" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="11">
         <f t="shared" ref="A3:A6" si="0">ROW(B3) - 2</f>
         <v>1</v>
@@ -2245,17 +2274,17 @@
       <c r="C3" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="10" t="s">
+        <v>337</v>
+      </c>
+      <c r="E3" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="F3" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="F3" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>59</v>
+      <c r="G3" s="12" t="b">
+        <v>1</v>
       </c>
       <c r="H3" s="12" t="s">
         <v>59</v>
@@ -2263,100 +2292,103 @@
       <c r="I3" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="J3" s="20">
+      <c r="J3" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="K3" s="20">
         <v>6672</v>
       </c>
-      <c r="K3" s="12"/>
-      <c r="M3" s="10"/>
-      <c r="O3" s="11" t="s">
+      <c r="L3" s="12"/>
+      <c r="N3" s="10"/>
+      <c r="P3" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="P3" s="11" t="s">
+      <c r="Q3" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="Q3" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="R3" s="11" t="s">
+      <c r="R3" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="S3" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="S3" s="11" t="s">
+      <c r="T3" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="T3" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="U3" s="11" t="s">
+      <c r="U3" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="V3" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="V3" s="11" t="s">
+      <c r="W3" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="W3" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="X3" s="11" t="s">
+      <c r="X3" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y3" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="Y3" s="12" t="s">
+      <c r="Z3" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="Z3" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA3" s="12" t="s">
+      <c r="AA3" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB3" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="AB3" s="12" t="s">
+      <c r="AC3" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="AC3" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD3" s="11" t="s">
+      <c r="AD3" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AE3" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="AE3" s="11" t="s">
+      <c r="AF3" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="AF3" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG3" s="11" t="s">
+      <c r="AG3" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH3" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="AH3" s="11" t="s">
+      <c r="AI3" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="AI3" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AJ3" s="11" t="s">
+      <c r="AJ3" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK3" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="AK3" s="11" t="s">
+      <c r="AL3" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="AL3" s="11" t="s">
+      <c r="AM3" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="AM3" s="11" t="b">
+      <c r="AN3" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="AN3" s="11" t="s">
+      <c r="AO3" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="AR3" s="11" t="s">
+      <c r="AS3" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="AS3" s="11" t="s">
+      <c r="AT3" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="AT3" s="11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:49" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AU3" s="11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:50" ht="32.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -2367,137 +2399,138 @@
       <c r="C4" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1"/>
+      <c r="E4" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="F4" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="F4" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>81</v>
+      <c r="G4" s="12" t="b">
+        <v>1</v>
       </c>
       <c r="H4" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="J4" s="15">
+      <c r="J4" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K4" s="15">
         <v>525</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>83</v>
       </c>
-      <c r="M4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N4" t="s">
+      <c r="N4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O4" t="s">
         <v>84</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>85</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>86</v>
       </c>
-      <c r="Q4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="R4" t="s">
+      <c r="R4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="S4" t="s">
         <v>87</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>88</v>
       </c>
-      <c r="T4" t="b">
-        <v>1</v>
-      </c>
-      <c r="X4" t="s">
+      <c r="U4" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y4" t="s">
         <v>89</v>
       </c>
-      <c r="Y4" s="2" t="s">
+      <c r="Z4" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="Z4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA4" s="2" t="s">
+      <c r="AA4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB4" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="AB4" s="2" t="s">
+      <c r="AC4" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AC4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD4" t="s">
+      <c r="AD4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AE4" t="s">
         <v>91</v>
       </c>
-      <c r="AE4" t="s">
+      <c r="AF4" t="s">
         <v>69</v>
       </c>
-      <c r="AF4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG4" t="s">
+      <c r="AG4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH4" t="s">
         <v>92</v>
       </c>
-      <c r="AH4" t="s">
+      <c r="AI4" t="s">
         <v>86</v>
       </c>
-      <c r="AI4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AJ4" t="s">
+      <c r="AJ4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK4" t="s">
         <v>71</v>
       </c>
-      <c r="AK4" t="s">
+      <c r="AL4" t="s">
         <v>93</v>
       </c>
-      <c r="AL4" t="s">
+      <c r="AM4" t="s">
         <v>94</v>
       </c>
-      <c r="AM4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AN4" t="s">
+      <c r="AN4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO4" t="s">
         <v>95</v>
       </c>
-      <c r="AO4" t="s">
+      <c r="AP4" t="s">
         <v>96</v>
       </c>
-      <c r="AP4" t="s">
+      <c r="AQ4" t="s">
         <v>97</v>
       </c>
-      <c r="AQ4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AR4" t="s">
+      <c r="AR4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS4" t="s">
         <v>98</v>
       </c>
-      <c r="AS4" t="s">
+      <c r="AT4" t="s">
         <v>99</v>
       </c>
-      <c r="AT4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AU4" t="s">
+      <c r="AU4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AV4" t="s">
         <v>100</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AW4" t="s">
         <v>69</v>
       </c>
-      <c r="AW4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:49" ht="42.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AX4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:50" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -2508,111 +2541,112 @@
       <c r="C5" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1"/>
+      <c r="E5" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="F5" s="12" t="s">
         <v>329</v>
       </c>
-      <c r="F5" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>104</v>
+      <c r="G5" s="12" t="b">
+        <v>1</v>
       </c>
       <c r="H5" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="M5" s="1"/>
-      <c r="O5" t="s">
+      <c r="J5" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="N5" s="1"/>
+      <c r="P5" t="s">
         <v>105</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>69</v>
       </c>
-      <c r="Q5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="R5" t="s">
+      <c r="R5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="S5" t="s">
         <v>106</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>88</v>
       </c>
-      <c r="T5" t="b">
-        <v>1</v>
-      </c>
-      <c r="X5" t="s">
+      <c r="U5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y5" t="s">
         <v>107</v>
       </c>
-      <c r="Y5" s="2" t="s">
+      <c r="Z5" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="Z5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA5" s="2" t="s">
+      <c r="AA5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB5" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="AB5" s="2" t="s">
+      <c r="AC5" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="AC5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD5" t="s">
+      <c r="AD5" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AE5" t="s">
         <v>109</v>
       </c>
-      <c r="AE5" t="s">
+      <c r="AF5" t="s">
         <v>69</v>
       </c>
-      <c r="AF5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG5" t="s">
+      <c r="AG5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH5" t="s">
         <v>105</v>
       </c>
-      <c r="AH5" t="s">
+      <c r="AI5" t="s">
         <v>69</v>
       </c>
-      <c r="AI5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AJ5" t="s">
+      <c r="AJ5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK5" t="s">
         <v>71</v>
       </c>
-      <c r="AK5" t="s">
+      <c r="AL5" t="s">
         <v>110</v>
       </c>
-      <c r="AL5" t="s">
+      <c r="AM5" t="s">
         <v>111</v>
       </c>
-      <c r="AM5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AN5" t="s">
+      <c r="AN5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO5" t="s">
         <v>112</v>
       </c>
-      <c r="AO5" t="s">
+      <c r="AP5" t="s">
         <v>113</v>
       </c>
-      <c r="AP5" t="s">
+      <c r="AQ5" t="s">
         <v>114</v>
       </c>
-      <c r="AQ5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AT5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AU5" t="s">
+      <c r="AR5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AU5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AV5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="6" spans="1:49" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:50" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -2623,116 +2657,117 @@
       <c r="C6" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="1"/>
+      <c r="E6" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="F6" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="F6" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>120</v>
+      <c r="G6" s="12" t="b">
+        <v>1</v>
       </c>
       <c r="H6" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="K6" s="15">
         <v>3713</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="L6" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>83</v>
       </c>
-      <c r="M6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O6" t="s">
+      <c r="N6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P6" t="s">
         <v>122</v>
       </c>
-      <c r="P6" t="s">
+      <c r="Q6" t="s">
         <v>123</v>
       </c>
-      <c r="Q6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="R6" t="s">
+      <c r="R6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="S6" t="s">
         <v>124</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>88</v>
       </c>
-      <c r="T6" t="b">
-        <v>1</v>
-      </c>
-      <c r="X6" t="s">
+      <c r="U6" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y6" t="s">
         <v>125</v>
       </c>
-      <c r="Y6" s="2" t="s">
+      <c r="Z6" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="Z6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA6" s="2" t="s">
+      <c r="AA6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB6" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="AB6" s="2" t="s">
+      <c r="AC6" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AC6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG6" t="s">
+      <c r="AD6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH6" t="s">
         <v>122</v>
       </c>
-      <c r="AH6" t="s">
+      <c r="AI6" t="s">
         <v>123</v>
       </c>
-      <c r="AI6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AJ6" t="s">
+      <c r="AJ6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK6" t="s">
         <v>71</v>
       </c>
-      <c r="AK6" t="s">
+      <c r="AL6" t="s">
         <v>127</v>
       </c>
-      <c r="AL6" t="s">
+      <c r="AM6" t="s">
         <v>128</v>
       </c>
-      <c r="AM6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AN6" t="s">
+      <c r="AN6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO6" t="s">
         <v>129</v>
       </c>
-      <c r="AO6" t="s">
+      <c r="AP6" t="s">
         <v>130</v>
       </c>
-      <c r="AP6" t="s">
+      <c r="AQ6" t="s">
         <v>69</v>
       </c>
-      <c r="AQ6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AU6" t="s">
+      <c r="AR6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AV6" t="s">
         <v>131</v>
       </c>
-      <c r="AV6" t="s">
+      <c r="AW6" t="s">
         <v>69</v>
       </c>
-      <c r="AW6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:49" ht="45" x14ac:dyDescent="0.25">
+      <c r="AX6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:50" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7">
         <f t="shared" ref="A7:A12" si="1">ROW(B7) - 2</f>
         <v>5</v>
@@ -2743,116 +2778,117 @@
       <c r="C7" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1"/>
+      <c r="E7" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="F7" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="F7" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>81</v>
+      <c r="G7" s="12" t="b">
+        <v>1</v>
       </c>
       <c r="H7" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K7" s="15">
         <v>525</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="L7" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>83</v>
       </c>
-      <c r="M7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O7" t="s">
+      <c r="N7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P7" t="s">
         <v>135</v>
       </c>
-      <c r="P7" t="s">
+      <c r="Q7" t="s">
         <v>86</v>
       </c>
-      <c r="Q7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="R7" s="15" t="s">
+      <c r="R7" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="S7" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="S7" s="15" t="s">
+      <c r="T7" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="T7" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="X7" s="15" t="s">
+      <c r="U7" s="14" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="Y7" s="15" t="s">
+      <c r="Z7" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="Z7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA7" s="2" t="s">
+      <c r="AA7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB7" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="AB7" s="2" t="s">
+      <c r="AC7" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AC7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD7" s="15" t="s">
+      <c r="AD7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AE7" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="AE7" s="15" t="s">
+      <c r="AF7" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="AF7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG7" t="s">
+      <c r="AG7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH7" t="s">
         <v>135</v>
       </c>
-      <c r="AH7" t="s">
+      <c r="AI7" t="s">
         <v>86</v>
       </c>
-      <c r="AI7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AJ7" t="s">
+      <c r="AJ7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK7" t="s">
         <v>71</v>
       </c>
-      <c r="AK7" t="s">
+      <c r="AL7" t="s">
         <v>93</v>
       </c>
-      <c r="AL7" t="s">
+      <c r="AM7" t="s">
         <v>94</v>
       </c>
-      <c r="AM7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AN7" t="s">
+      <c r="AN7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO7" t="s">
         <v>95</v>
       </c>
-      <c r="AO7" t="s">
+      <c r="AP7" t="s">
         <v>96</v>
       </c>
-      <c r="AP7" t="s">
+      <c r="AQ7" t="s">
         <v>97</v>
       </c>
-      <c r="AQ7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:49" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AR7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:50" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <f t="shared" si="1"/>
         <v>6</v>
@@ -2863,17 +2899,15 @@
       <c r="C8" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1"/>
+      <c r="E8" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="F8" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="F8" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>144</v>
+      <c r="G8" s="12" t="b">
+        <v>1</v>
       </c>
       <c r="H8" s="12" t="s">
         <v>144</v>
@@ -2881,110 +2915,113 @@
       <c r="I8" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="J8" s="15">
+      <c r="J8" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="K8" s="15">
         <v>5386</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="L8" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>83</v>
       </c>
-      <c r="M8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N8" t="s">
+      <c r="N8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O8" t="s">
         <v>146</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
         <v>147</v>
       </c>
-      <c r="P8" t="s">
+      <c r="Q8" t="s">
         <v>86</v>
       </c>
-      <c r="Q8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="R8" t="s">
+      <c r="R8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="S8" t="s">
         <v>148</v>
       </c>
-      <c r="S8" t="s">
+      <c r="T8" t="s">
         <v>88</v>
       </c>
-      <c r="T8" t="b">
-        <v>1</v>
-      </c>
-      <c r="X8" t="s">
+      <c r="U8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y8" t="s">
         <v>149</v>
       </c>
-      <c r="Y8" s="2" t="s">
+      <c r="Z8" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="Z8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA8" s="2" t="s">
+      <c r="AA8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB8" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="AB8" s="2" t="s">
+      <c r="AC8" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AC8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD8" t="s">
+      <c r="AD8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AE8" t="s">
         <v>151</v>
       </c>
-      <c r="AE8" t="s">
+      <c r="AF8" t="s">
         <v>69</v>
       </c>
-      <c r="AF8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG8" t="s">
+      <c r="AG8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH8" t="s">
         <v>147</v>
       </c>
-      <c r="AH8" t="s">
+      <c r="AI8" t="s">
         <v>86</v>
       </c>
-      <c r="AI8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AJ8" t="s">
+      <c r="AJ8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK8" t="s">
         <v>71</v>
       </c>
-      <c r="AK8" t="s">
+      <c r="AL8" t="s">
         <v>152</v>
       </c>
-      <c r="AL8" t="s">
+      <c r="AM8" t="s">
         <v>153</v>
       </c>
-      <c r="AM8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AN8" t="s">
+      <c r="AN8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO8" t="s">
         <v>154</v>
       </c>
-      <c r="AO8" t="s">
+      <c r="AP8" t="s">
         <v>155</v>
       </c>
-      <c r="AP8" t="s">
+      <c r="AQ8" t="s">
         <v>69</v>
       </c>
-      <c r="AQ8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AU8" t="s">
+      <c r="AR8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AV8" t="s">
         <v>156</v>
       </c>
-      <c r="AV8" t="s">
+      <c r="AW8" t="s">
         <v>69</v>
       </c>
-      <c r="AW8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:49" ht="55.35" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AX8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:50" ht="55.35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <f t="shared" si="1"/>
         <v>7</v>
@@ -2995,119 +3032,120 @@
       <c r="C9" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="1"/>
+      <c r="E9" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="F9" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="F9" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>161</v>
+      <c r="G9" s="12" t="b">
+        <v>1</v>
       </c>
       <c r="H9" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="J9" s="15">
+      <c r="J9" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="K9" s="15">
         <v>2735</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="L9" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>83</v>
       </c>
-      <c r="M9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N9" t="s">
+      <c r="N9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O9" t="s">
         <v>163</v>
       </c>
-      <c r="O9" t="s">
+      <c r="P9" t="s">
         <v>164</v>
       </c>
-      <c r="P9" t="s">
+      <c r="Q9" t="s">
         <v>165</v>
       </c>
-      <c r="Q9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="R9" t="s">
+      <c r="R9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="S9" t="s">
         <v>166</v>
       </c>
-      <c r="S9" t="s">
+      <c r="T9" t="s">
         <v>88</v>
       </c>
-      <c r="T9" t="b">
-        <v>1</v>
-      </c>
-      <c r="X9" t="s">
+      <c r="U9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y9" t="s">
         <v>167</v>
       </c>
-      <c r="Y9" s="2" t="s">
+      <c r="Z9" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="Z9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA9" s="2" t="s">
+      <c r="AA9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB9" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="AB9" s="2" t="s">
+      <c r="AC9" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AC9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG9" t="s">
+      <c r="AD9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH9" t="s">
         <v>164</v>
       </c>
-      <c r="AH9" t="s">
+      <c r="AI9" t="s">
         <v>169</v>
       </c>
-      <c r="AI9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AJ9" t="s">
+      <c r="AJ9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK9" t="s">
         <v>71</v>
       </c>
-      <c r="AK9" t="s">
+      <c r="AL9" t="s">
         <v>170</v>
       </c>
-      <c r="AL9" t="s">
+      <c r="AM9" t="s">
         <v>171</v>
       </c>
-      <c r="AM9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AN9" t="s">
+      <c r="AN9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO9" t="s">
         <v>172</v>
       </c>
-      <c r="AO9" t="s">
+      <c r="AP9" t="s">
         <v>173</v>
       </c>
-      <c r="AP9" t="s">
+      <c r="AQ9" t="s">
         <v>97</v>
       </c>
-      <c r="AQ9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AU9" t="s">
+      <c r="AR9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AV9" t="s">
         <v>174</v>
       </c>
-      <c r="AV9" t="s">
+      <c r="AW9" t="s">
         <v>69</v>
       </c>
-      <c r="AW9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:49" ht="44.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AX9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:50" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <f t="shared" si="1"/>
         <v>8</v>
@@ -3118,122 +3156,123 @@
       <c r="C10" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="1"/>
+      <c r="E10" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="F10" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="F10" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>161</v>
+      <c r="G10" s="12" t="b">
+        <v>1</v>
       </c>
       <c r="H10" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="J10" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="L10" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>83</v>
       </c>
-      <c r="M10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O10" t="s">
+      <c r="N10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P10" t="s">
         <v>180</v>
       </c>
-      <c r="P10" t="s">
+      <c r="Q10" t="s">
         <v>69</v>
       </c>
-      <c r="Q10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="R10" t="s">
+      <c r="R10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="S10" t="s">
         <v>181</v>
       </c>
-      <c r="S10" t="s">
+      <c r="T10" t="s">
         <v>88</v>
       </c>
-      <c r="T10" t="b">
-        <v>1</v>
-      </c>
-      <c r="X10" t="s">
+      <c r="U10" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y10" t="s">
         <v>182</v>
       </c>
-      <c r="Y10" s="2" t="s">
+      <c r="Z10" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="Z10" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA10" t="s">
+      <c r="AA10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB10" t="s">
         <v>183</v>
       </c>
-      <c r="AB10" s="2" t="s">
+      <c r="AC10" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AC10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD10" t="s">
+      <c r="AD10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AE10" t="s">
         <v>184</v>
       </c>
-      <c r="AE10" t="s">
+      <c r="AF10" t="s">
         <v>69</v>
       </c>
-      <c r="AF10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG10" t="s">
+      <c r="AG10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH10" t="s">
         <v>180</v>
       </c>
-      <c r="AH10" t="s">
+      <c r="AI10" t="s">
         <v>69</v>
       </c>
-      <c r="AI10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AJ10" t="s">
+      <c r="AJ10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK10" t="s">
         <v>71</v>
       </c>
-      <c r="AK10" t="s">
+      <c r="AL10" t="s">
         <v>185</v>
       </c>
-      <c r="AL10" t="s">
+      <c r="AM10" t="s">
         <v>186</v>
       </c>
-      <c r="AM10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AN10" t="s">
+      <c r="AN10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO10" t="s">
         <v>187</v>
       </c>
-      <c r="AO10" t="s">
+      <c r="AP10" t="s">
         <v>313</v>
       </c>
-      <c r="AP10" t="s">
+      <c r="AQ10" t="s">
         <v>314</v>
       </c>
-      <c r="AQ10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AU10" t="s">
+      <c r="AR10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AV10" t="s">
         <v>315</v>
       </c>
-      <c r="AV10" t="s">
+      <c r="AW10" t="s">
         <v>69</v>
       </c>
-      <c r="AW10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:49" ht="45" x14ac:dyDescent="0.25">
+      <c r="AX10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:50" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11">
         <f t="shared" si="1"/>
         <v>9</v>
@@ -3244,137 +3283,140 @@
       <c r="C11" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="10" t="s">
+        <v>337</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="F11" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="F11" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>59</v>
+      <c r="G11" s="12" t="b">
+        <v>1</v>
       </c>
       <c r="H11" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="J11" s="15">
+      <c r="J11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="K11" s="15">
         <v>6672</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="L11" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>83</v>
       </c>
-      <c r="M11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N11" s="2" t="s">
+      <c r="N11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O11" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="O11" s="12" t="s">
+      <c r="P11" s="12" t="s">
         <v>190</v>
       </c>
-      <c r="P11" t="s">
+      <c r="Q11" t="s">
         <v>192</v>
       </c>
-      <c r="Q11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="R11" s="2" t="s">
+      <c r="R11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="S11" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="S11" s="11" t="s">
+      <c r="T11" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="T11" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="U11" s="11" t="s">
+      <c r="U11" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="V11" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="V11" s="11" t="s">
+      <c r="W11" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="W11" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="X11" s="2" t="s">
+      <c r="X11" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y11" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="Y11" s="12" t="s">
+      <c r="Z11" s="12" t="s">
         <v>194</v>
       </c>
-      <c r="Z11" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA11" s="2" t="s">
+      <c r="AA11" s="12" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB11" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="AB11" s="21" t="s">
+      <c r="AC11" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="AC11" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD11" s="12" t="s">
+      <c r="AD11" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AE11" s="12" t="s">
         <v>198</v>
       </c>
-      <c r="AE11" s="11" t="s">
+      <c r="AF11" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="AF11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG11" t="s">
+      <c r="AG11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH11" t="s">
         <v>190</v>
       </c>
-      <c r="AH11" t="s">
+      <c r="AI11" t="s">
         <v>192</v>
       </c>
-      <c r="AI11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AJ11" t="s">
+      <c r="AJ11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK11" t="s">
         <v>71</v>
       </c>
-      <c r="AK11" s="11" t="s">
+      <c r="AL11" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="AL11" s="11" t="s">
+      <c r="AM11" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="AM11" s="11" t="b">
+      <c r="AN11" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="AN11" s="11" t="s">
+      <c r="AO11" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="AR11" t="s">
+      <c r="AS11" t="s">
         <v>75</v>
       </c>
-      <c r="AS11" t="s">
+      <c r="AT11" t="s">
         <v>76</v>
       </c>
-      <c r="AT11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AU11" t="s">
+      <c r="AU11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AV11" t="s">
         <v>199</v>
       </c>
-      <c r="AV11" t="s">
+      <c r="AW11" t="s">
         <v>316</v>
       </c>
-      <c r="AW11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:49" ht="30" x14ac:dyDescent="0.25">
+      <c r="AX11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:50" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12">
         <f t="shared" si="1"/>
         <v>10</v>
@@ -3385,17 +3427,15 @@
       <c r="C12" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="1"/>
+      <c r="E12" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="F12" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="F12" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>203</v>
+      <c r="G12" s="12" t="b">
+        <v>1</v>
       </c>
       <c r="H12" s="12" t="s">
         <v>203</v>
@@ -3403,34 +3443,37 @@
       <c r="I12" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="J12" s="15">
+      <c r="J12" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="K12" s="15">
         <v>7098</v>
       </c>
-      <c r="K12" s="2" t="s">
+      <c r="L12" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>83</v>
       </c>
-      <c r="M12" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N12" s="2" t="s">
+      <c r="N12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O12" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="O12" s="2" t="s">
+      <c r="P12" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="P12" t="s">
+      <c r="Q12" t="s">
         <v>69</v>
       </c>
-      <c r="Q12" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC12" s="1"/>
-      <c r="AM12" s="1"/>
-    </row>
-    <row r="13" spans="1:49" ht="45" x14ac:dyDescent="0.25">
+      <c r="R12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD12" s="1"/>
+      <c r="AN12" s="1"/>
+    </row>
+    <row r="13" spans="1:50" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13">
         <f>ROW(B13) - 2</f>
         <v>11</v>
@@ -3441,17 +3484,15 @@
       <c r="C13" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="1"/>
+      <c r="E13" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="F13" s="12" t="s">
         <v>208</v>
       </c>
-      <c r="F13" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" s="12" t="s">
-        <v>209</v>
+      <c r="G13" s="12" t="b">
+        <v>1</v>
       </c>
       <c r="H13" s="12" t="s">
         <v>209</v>
@@ -3459,98 +3500,101 @@
       <c r="I13" s="12" t="s">
         <v>209</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="J13" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="L13" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>83</v>
       </c>
-      <c r="M13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="N13" s="2" t="s">
+      <c r="N13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="O13" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="O13" t="s">
+      <c r="P13" t="s">
         <v>210</v>
       </c>
-      <c r="P13" t="s">
+      <c r="Q13" t="s">
         <v>317</v>
       </c>
-      <c r="Q13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="R13" t="s">
+      <c r="R13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="S13" t="s">
         <v>321</v>
       </c>
-      <c r="S13" t="s">
+      <c r="T13" t="s">
         <v>194</v>
       </c>
-      <c r="T13" t="b">
-        <v>1</v>
-      </c>
-      <c r="X13" t="s">
+      <c r="U13" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y13" t="s">
         <v>322</v>
       </c>
-      <c r="Y13" s="2" t="s">
+      <c r="Z13" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="Z13" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA13" s="2" t="s">
+      <c r="AA13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB13" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="AB13" s="12" t="s">
+      <c r="AC13" s="12" t="s">
         <v>194</v>
       </c>
-      <c r="AC13" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG13" t="s">
+      <c r="AD13" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH13" t="s">
         <v>210</v>
       </c>
-      <c r="AH13" t="s">
+      <c r="AI13" t="s">
         <v>317</v>
       </c>
-      <c r="AI13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AJ13" t="s">
+      <c r="AJ13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK13" t="s">
         <v>71</v>
       </c>
-      <c r="AK13" t="s">
+      <c r="AL13" t="s">
         <v>324</v>
       </c>
-      <c r="AL13" t="s">
+      <c r="AM13" t="s">
         <v>171</v>
       </c>
-      <c r="AM13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AN13" t="s">
+      <c r="AN13" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO13" t="s">
         <v>325</v>
       </c>
-      <c r="AO13" t="s">
+      <c r="AP13" t="s">
         <v>326</v>
       </c>
-      <c r="AP13" t="s">
+      <c r="AQ13" t="s">
         <v>327</v>
       </c>
-      <c r="AQ13" t="b">
-        <v>1</v>
-      </c>
-      <c r="AU13" s="2" t="s">
+      <c r="AR13" t="b">
+        <v>1</v>
+      </c>
+      <c r="AV13" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="AV13" t="s">
+      <c r="AW13" t="s">
         <v>69</v>
       </c>
-      <c r="AW13" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:49" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AX13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:50" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <f>ROW(B14) - 2</f>
         <v>12</v>
@@ -3561,17 +3605,15 @@
       <c r="C14" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="1"/>
+      <c r="E14" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="F14" s="12" t="s">
         <v>215</v>
       </c>
-      <c r="F14" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G14" s="12" t="s">
-        <v>216</v>
+      <c r="G14" s="12" t="b">
+        <v>1</v>
       </c>
       <c r="H14" s="12" t="s">
         <v>216</v>
@@ -3579,105 +3621,109 @@
       <c r="I14" s="12" t="s">
         <v>216</v>
       </c>
-      <c r="K14" s="2" t="s">
+      <c r="J14" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="L14" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="L14" t="s">
+      <c r="M14" t="s">
         <v>218</v>
       </c>
-      <c r="M14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O14" t="s">
+      <c r="N14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="P14" t="s">
         <v>217</v>
       </c>
-      <c r="P14" t="s">
+      <c r="Q14" t="s">
         <v>218</v>
       </c>
-      <c r="Q14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="R14" t="s">
+      <c r="R14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="S14" t="s">
         <v>219</v>
       </c>
-      <c r="S14" t="s">
+      <c r="T14" t="s">
         <v>88</v>
       </c>
-      <c r="T14" t="b">
-        <v>1</v>
-      </c>
-      <c r="X14" t="s">
+      <c r="U14" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y14" t="s">
         <v>220</v>
       </c>
-      <c r="Y14" s="2" t="s">
+      <c r="Z14" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="Z14" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AA14" s="2" t="s">
+      <c r="AA14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB14" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="AB14" s="2" t="s">
+      <c r="AC14" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="AC14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD14" t="s">
+      <c r="AD14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AE14" t="s">
         <v>222</v>
       </c>
-      <c r="AE14" s="11" t="s">
+      <c r="AF14" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="AF14" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG14" t="s">
+      <c r="AG14" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH14" t="s">
         <v>217</v>
       </c>
-      <c r="AH14" t="s">
+      <c r="AI14" t="s">
         <v>218</v>
       </c>
-      <c r="AI14" t="b">
-        <v>1</v>
-      </c>
-      <c r="AJ14" t="s">
+      <c r="AJ14" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK14" t="s">
         <v>71</v>
       </c>
-      <c r="AK14" t="s">
+      <c r="AL14" t="s">
         <v>223</v>
       </c>
-      <c r="AL14" t="s">
+      <c r="AM14" t="s">
         <v>224</v>
       </c>
-      <c r="AM14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AN14" t="s">
+      <c r="AN14" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO14" t="s">
         <v>225</v>
       </c>
-      <c r="AO14" t="s">
+      <c r="AP14" t="s">
         <v>226</v>
       </c>
-      <c r="AP14" t="s">
+      <c r="AQ14" t="s">
         <v>227</v>
       </c>
-      <c r="AQ14" t="b">
-        <v>1</v>
-      </c>
-      <c r="AU14" t="s">
+      <c r="AR14" t="b">
+        <v>1</v>
+      </c>
+      <c r="AV14" t="s">
         <v>228</v>
       </c>
-      <c r="AV14" t="s">
+      <c r="AW14" t="s">
         <v>115</v>
       </c>
-      <c r="AW14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:49" x14ac:dyDescent="0.25">
+      <c r="AX14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A15">
+        <f>ROW(B15) - 2</f>
         <v>13</v>
       </c>
       <c r="B15" t="s">
@@ -3686,82 +3732,106 @@
       <c r="C15" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="1"/>
+      <c r="E15" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="E15" s="12" t="s">
+      <c r="F15" s="12" t="s">
         <v>208</v>
       </c>
-      <c r="F15" s="12" t="b">
+      <c r="G15" s="12" t="b">
         <v>0</v>
-      </c>
-      <c r="G15" s="12" t="s">
-        <v>209</v>
       </c>
       <c r="H15" s="12" t="s">
         <v>209</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="I15" s="12" t="s">
         <v>209</v>
       </c>
-      <c r="M15" s="1"/>
-      <c r="Q15" s="1"/>
-      <c r="AC15" s="1"/>
-      <c r="AM15" s="1"/>
+      <c r="J15" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="N15" s="1"/>
+      <c r="R15" s="1"/>
+      <c r="AD15" s="1"/>
+      <c r="AN15" s="1"/>
+    </row>
+    <row r="16" spans="1:50" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <f>ROW(B16) - 2</f>
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>333</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="D16" s="1"/>
+      <c r="E16" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="G16" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="N16" s="1"/>
+      <c r="R16" s="1"/>
+      <c r="AD16" s="1"/>
+      <c r="AN16" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="AG1:AW1"/>
-    <mergeCell ref="D1:M1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="R1:AC1"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="AD1:AF1"/>
+    <mergeCell ref="AH1:AX1"/>
+    <mergeCell ref="E1:N1"/>
+    <mergeCell ref="S1:AD1"/>
+    <mergeCell ref="P1:R1"/>
+    <mergeCell ref="AE1:AG1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A2" location="DEF_INDEX" display="INDEX" xr:uid="{0B4D13DD-2ADD-4A2C-B155-A44799CAFB5D}"/>
     <hyperlink ref="B2" location="DEF_NAME" display="NAME" xr:uid="{DFA26519-DA67-4585-92D4-B8B4ADD88299}"/>
     <hyperlink ref="C2" location="DEF_ID" display="ID" xr:uid="{A76C0444-0C5B-465B-A613-350B7921D272}"/>
-    <hyperlink ref="D2" location="DEF_WATERSHED_BOUNDARY_DATABASE_PATH" display="WATERSHED_BOUNDARY_DATABASE_PATH" xr:uid="{957822AC-FA53-4CB2-86C1-AA3A9649CA15}"/>
-    <hyperlink ref="E2" location="DEF_WATERSHED_BOUNDARY_LAYER_NAME" display="WATERSHED_BOUNDARY_LAYER_NAME" xr:uid="{0DBD66A9-7022-493C-8E9A-ECE4EC2DAC6C}"/>
-    <hyperlink ref="F2" location="DEF_IS_SHAREPOINT_PATH_WATERSHED_BOUNDARY" display="IS_SHAREPOINT_PATH_WATERSHED_BOUNDARY" xr:uid="{65941A0B-8FA5-41D4-BEBD-7C8D23AF17B3}"/>
-    <hyperlink ref="J2" location="DEF_WATERSHED_EXIT_POINT_INDEX" display="WATERSHED_EXIT_POINT_INDEX" xr:uid="{B4DABB88-D07E-4344-8A98-833B79BCB66A}"/>
-    <hyperlink ref="K2" location="DEF_GIS_PREPROCESSING_SPREADSHEET_PATH" display="GIS_PREPROCESSING_SPREADSHEET_PATH" xr:uid="{2D94ADE4-7566-4CF3-9304-65D819D5331E}"/>
-    <hyperlink ref="L2" location="DEF_GIS_PREPROCESSING_WORKSHEET_NAME" display="GIS_PREPROCESSING_WORKSHEET_NAME" xr:uid="{9769E079-549D-481F-A5C9-05B7BD9055AB}"/>
-    <hyperlink ref="M2" location="DEF_IS_SHAREPOINT_PATH_GIS_PREPROCESSING_SPREADSHEET" display="IS_SHAREPOINT_PATH_GIS_PREPROCESSING_SPREADSHEET" xr:uid="{B944ED1B-FE52-492B-B5BF-75E7EBB4D560}"/>
-    <hyperlink ref="R2" location="DEF_QAQC_UNIT_CONVERSION_ERRORS_SPREADSHEET_PATH" display="QAQC_UNIT_CONVERSION_ERRORS_SPREADSHEET_PATH" xr:uid="{40780C1A-FFC4-4031-B7A5-940F297B6694}"/>
-    <hyperlink ref="S2" location="DEF_QAQC_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME" display="QAQC_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME" xr:uid="{61F0092E-1844-4B06-BAB7-CE62ADABA8B2}"/>
-    <hyperlink ref="T2" location="DEF_IS_SHAREPOINT_PATH_QAQC_UNIT_CONVERSION_ERRORS_SPREADSHEET" display="IS_SHAREPOINT_PATH_QAQC_UNIT_CONVERSION_ERRORS_SPREADSHEET" xr:uid="{AE38E335-1793-4E31-B09C-DA10F3D50109}"/>
-    <hyperlink ref="X2" location="DEF_QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET_PATH" display="QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET_PATH" xr:uid="{CF7C45B0-BD5F-47F7-85FE-3F5D21FB09E5}"/>
-    <hyperlink ref="Y2" location="DEF_QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME" display="QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME" xr:uid="{58CB88C4-DBA4-4D9F-AD1D-DFCFD566F2B2}"/>
-    <hyperlink ref="Z2" location="DEF_IS_SHAREPOINT_PATH_QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET" display="IS_SHAREPOINT_PATH_QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET" xr:uid="{4105506E-B958-4B57-825A-CAC9B8022A7D}"/>
-    <hyperlink ref="AA2" location="DEF_QAQC_DUPLICATE_REPORTING_SPREADSHEET_PATH" display="QAQC_DUPLICATE_REPORTING_SPREADSHEET_PATH" xr:uid="{E1EDFB86-7204-4510-89AE-5ACE03491666}"/>
-    <hyperlink ref="AB2" location="DEF_QAQC_DUPLICATE_REPORTING_WORKSHEET_NAME" display="QAQC_DUPLICATE_REPORTING_WORKSHEET_NAME" xr:uid="{F9692A09-4738-4D34-B93C-CA7CC29D7F7C}"/>
-    <hyperlink ref="AC2" location="DEF_IS_SHAREPOINT_PATH_QAQC_DUPLICATE_REPORTING_SPREADSHEET" display="IS_SHAREPOINT_PATH_QAQC_DUPLICATE_REPORTING_SPREADSHEET" xr:uid="{BF670201-91D3-4F29-A971-6BB04CD1B279}"/>
-    <hyperlink ref="O2" location="DEF_POD_APPLICATION_NUMBER_SPREADSHEET_PATH" display="POD_APPLICATION_NUMBER_SPREADSHEET_PATH" xr:uid="{E186013E-9D32-41EF-B225-6D25FB3EFEB4}"/>
-    <hyperlink ref="P2" location="DEF_POD_APPLICATION_NUMBER_WORKSHEET_NAME" display="POD_APPLICATION_NUMBER_WORKSHEET_NAME" xr:uid="{7E26A27A-1026-49D8-A2BD-4D383B725B71}"/>
-    <hyperlink ref="Q2" location="DEF_IS_SHAREPOINT_PATH_POD_APPLICATION_NUMBER_SPREADSHEET" display="IS_SHAREPOINT_PATH_POD_APPLICATION_NUMBER_SPREADSHEET" xr:uid="{93445971-A6B3-4683-B9ED-4EC2649A5511}"/>
-    <hyperlink ref="G2" location="DEF_WATERSHED_COLUMN_SEARCH_STRING" display="WATERSHED_COLUMN_SEARCH_STRING" xr:uid="{3DA8109F-5025-460F-B94D-26E5003B13CB}"/>
-    <hyperlink ref="H2" location="DEF_SOURCE_NAME_COLUMN_SEARCH_STRING" display="SOURCE_NAME_COLUMN_SEARCH_STRING" xr:uid="{E57F2D8B-2DBA-41E6-BEEC-BC667116A809}"/>
-    <hyperlink ref="I2" location="DEF_TRIB_DESC_COLUMN_SEARCH_STRING" display="TRIB_DESC_COLUMN_SEARCH_STRING" xr:uid="{47538E7D-F5BD-4AF1-8BB9-7E954BEDDC7F}"/>
-    <hyperlink ref="W2" location="DEF_IS_SHAREPOINT_PATH_QAQC_MEASUREMENT_VALUES" display="IS_SHAREPOINT_PATH_QAQC_MEASUREMENT_VALUES" xr:uid="{2796F3B2-5B56-4C81-90CB-623697BE3815}"/>
-    <hyperlink ref="U2" location="DEF_QAQC_MEASUREMENT_VALUES_SPREADSHEET_PATH" display="QAQC_MEASUREMENT_VALUES_SPREADSHEET_PATH" xr:uid="{55003B0F-9F85-4F33-AE2A-F833A902756C}"/>
-    <hyperlink ref="V2" location="DEF_QAQC_MEASUREMENT_VALUES_SPREADSHEET_WORKSHEET_NAME" display="QAQC_MEASUREMENT_VALUES_SPREADSHEET_WORKSHEET_NAME" xr:uid="{A7CF35CA-94DC-43B7-BB79-1A436B41D0F3}"/>
-    <hyperlink ref="AK2" location="DEF_SUBBASIN_POLYGONS_DATABASE_PATH" display="SUBBASIN_POLYGONS_DATABASE_PATH" xr:uid="{C4C102A6-1FBB-4666-8B15-EFA18CA68908}"/>
-    <hyperlink ref="AL2" location="DEF_SUBBASIN_POLYGONS_LAYER_NAME" display="SUBBASIN_POLYGONS_LAYER_NAME" xr:uid="{DC257581-78C3-40E5-B24A-59C01F8231D3}"/>
-    <hyperlink ref="AM2" location="DEF_IS_SHAREPOINT_PATH_SUBBASIN_POLYGONS" display="IS_SHAREPOINT_PATH_SUBBASIN_POLYGONS" xr:uid="{77276DAA-B389-48F1-90C9-2EAD01AAA728}"/>
-    <hyperlink ref="AN2" location="DEF_SUBBASIN_FIELD_ID_NAMES" display="SUBBASIN_FIELD_ID_NAMES" xr:uid="{174AF97C-F07C-4970-BE83-486F3D0014FC}"/>
-    <hyperlink ref="AR2" location="DEF_SUBBASIN_MANUAL_ASSIGNMENT_SPREADSHEET_PATH" display="SUBBASIN_MANUAL_ASSIGNMENT_SPREADSHEET_PATH" xr:uid="{33EBA2E4-0FBA-48C7-8A43-AC6242821539}"/>
-    <hyperlink ref="AS2" location="DEF_SUBBASIN_MANUAL_ASSIGNMENT_WORKSHEET_NAME" display="SUBBASIN_MANUAL_ASSIGNMENT_WORKSHEET_NAME" xr:uid="{0B1DEE05-94E3-4E0D-96D7-B50063C21133}"/>
-    <hyperlink ref="AT2" location="IS_SHAREPOINT_PATH_SUBBASIN_MANUAL_ASSIGNMENT" display="IS_SHAREPOINT_PATH_SUBBASIN_MANUAL_ASSIGNMENT" xr:uid="{A29D92E3-255E-4AE3-AC73-92CCFC7FC661}"/>
-    <hyperlink ref="AD2" location="DEF_NA_REPORTS_SPREADSHEET_PATH" display="NA_REPORTS_SPREADSHEET_PATH" xr:uid="{B995A17C-FCF7-4ED1-933D-00BE31FADD66}"/>
-    <hyperlink ref="AE2" location="DEF_NA_REPORTS_WORKSHEET_NAME" display="NA_REPORTS_WORKSHEET_NAME" xr:uid="{6A6A3F67-2FE2-4B33-9D75-BA533F9A3AB0}"/>
-    <hyperlink ref="AF2" location="DEF_IS_SHAREPOINT_PATH_NA_REPORTS_SPREADSHEET" display="IS_SHAREPOINT_PATH_NA_REPORTS_SPREADSHEET" xr:uid="{95415EA4-6F34-43DC-9BDB-548DF46BD083}"/>
-    <hyperlink ref="AO2" location="DEF_CONNECTIVITY_MATRIX_SPREADSHEET_PATH" display="CONNECTIVITY_MATRIX_SPREADSHEET_PATH" xr:uid="{5E74688E-EA6A-4805-B667-1AAC623445B0}"/>
-    <hyperlink ref="AP2" location="DEF_CONNECTIVITY_MATRIX_WORKSHEET_NAME" display="CONNECTIVITY_MATRIX_WORKSHEET_NAME" xr:uid="{6E1364E1-9CBE-4981-8009-6EF041C3D455}"/>
-    <hyperlink ref="AQ2" location="DEF_IS_SHAREPOINT_PATH_CONNECTIVITY_MATRIX_SPREADSHEET" display="IS_SHAREPOINT_PATH_CONNECTIVITY_MATRIX_SPREADSHEET" xr:uid="{81A63910-7028-4A75-8BDC-211C3A7D77B7}"/>
-    <hyperlink ref="N2" location="Dictionary!A1" display="EWRIMS_REPORTS_FOLDER_PATH" xr:uid="{8A43C4BA-14A9-4A97-B19F-C68BF3096FFB}"/>
+    <hyperlink ref="E2" location="DEF_WATERSHED_BOUNDARY_DATABASE_PATH" display="WATERSHED_BOUNDARY_DATABASE_PATH" xr:uid="{957822AC-FA53-4CB2-86C1-AA3A9649CA15}"/>
+    <hyperlink ref="F2" location="DEF_WATERSHED_BOUNDARY_LAYER_NAME" display="WATERSHED_BOUNDARY_LAYER_NAME" xr:uid="{0DBD66A9-7022-493C-8E9A-ECE4EC2DAC6C}"/>
+    <hyperlink ref="G2" location="DEF_IS_SHAREPOINT_PATH_WATERSHED_BOUNDARY" display="IS_SHAREPOINT_PATH_WATERSHED_BOUNDARY" xr:uid="{65941A0B-8FA5-41D4-BEBD-7C8D23AF17B3}"/>
+    <hyperlink ref="K2" location="DEF_WATERSHED_EXIT_POINT_INDEX" display="WATERSHED_EXIT_POINT_INDEX" xr:uid="{B4DABB88-D07E-4344-8A98-833B79BCB66A}"/>
+    <hyperlink ref="L2" location="DEF_GIS_PREPROCESSING_SPREADSHEET_PATH" display="GIS_PREPROCESSING_SPREADSHEET_PATH" xr:uid="{2D94ADE4-7566-4CF3-9304-65D819D5331E}"/>
+    <hyperlink ref="M2" location="DEF_GIS_PREPROCESSING_WORKSHEET_NAME" display="GIS_PREPROCESSING_WORKSHEET_NAME" xr:uid="{9769E079-549D-481F-A5C9-05B7BD9055AB}"/>
+    <hyperlink ref="N2" location="DEF_IS_SHAREPOINT_PATH_GIS_PREPROCESSING_SPREADSHEET" display="IS_SHAREPOINT_PATH_GIS_PREPROCESSING_SPREADSHEET" xr:uid="{B944ED1B-FE52-492B-B5BF-75E7EBB4D560}"/>
+    <hyperlink ref="S2" location="DEF_QAQC_UNIT_CONVERSION_ERRORS_SPREADSHEET_PATH" display="QAQC_UNIT_CONVERSION_ERRORS_SPREADSHEET_PATH" xr:uid="{40780C1A-FFC4-4031-B7A5-940F297B6694}"/>
+    <hyperlink ref="T2" location="DEF_QAQC_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME" display="QAQC_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME" xr:uid="{61F0092E-1844-4B06-BAB7-CE62ADABA8B2}"/>
+    <hyperlink ref="U2" location="DEF_IS_SHAREPOINT_PATH_QAQC_UNIT_CONVERSION_ERRORS_SPREADSHEET" display="IS_SHAREPOINT_PATH_QAQC_UNIT_CONVERSION_ERRORS_SPREADSHEET" xr:uid="{AE38E335-1793-4E31-B09C-DA10F3D50109}"/>
+    <hyperlink ref="Y2" location="DEF_QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET_PATH" display="QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET_PATH" xr:uid="{CF7C45B0-BD5F-47F7-85FE-3F5D21FB09E5}"/>
+    <hyperlink ref="Z2" location="DEF_QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME" display="QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME" xr:uid="{58CB88C4-DBA4-4D9F-AD1D-DFCFD566F2B2}"/>
+    <hyperlink ref="AA2" location="DEF_IS_SHAREPOINT_PATH_QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET" display="IS_SHAREPOINT_PATH_QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET" xr:uid="{4105506E-B958-4B57-825A-CAC9B8022A7D}"/>
+    <hyperlink ref="AB2" location="DEF_QAQC_DUPLICATE_REPORTING_SPREADSHEET_PATH" display="QAQC_DUPLICATE_REPORTING_SPREADSHEET_PATH" xr:uid="{E1EDFB86-7204-4510-89AE-5ACE03491666}"/>
+    <hyperlink ref="AC2" location="DEF_QAQC_DUPLICATE_REPORTING_WORKSHEET_NAME" display="QAQC_DUPLICATE_REPORTING_WORKSHEET_NAME" xr:uid="{F9692A09-4738-4D34-B93C-CA7CC29D7F7C}"/>
+    <hyperlink ref="AD2" location="DEF_IS_SHAREPOINT_PATH_QAQC_DUPLICATE_REPORTING_SPREADSHEET" display="IS_SHAREPOINT_PATH_QAQC_DUPLICATE_REPORTING_SPREADSHEET" xr:uid="{BF670201-91D3-4F29-A971-6BB04CD1B279}"/>
+    <hyperlink ref="P2" location="DEF_POD_APPLICATION_NUMBER_SPREADSHEET_PATH" display="POD_APPLICATION_NUMBER_SPREADSHEET_PATH" xr:uid="{E186013E-9D32-41EF-B225-6D25FB3EFEB4}"/>
+    <hyperlink ref="Q2" location="DEF_POD_APPLICATION_NUMBER_WORKSHEET_NAME" display="POD_APPLICATION_NUMBER_WORKSHEET_NAME" xr:uid="{7E26A27A-1026-49D8-A2BD-4D383B725B71}"/>
+    <hyperlink ref="R2" location="DEF_IS_SHAREPOINT_PATH_POD_APPLICATION_NUMBER_SPREADSHEET" display="IS_SHAREPOINT_PATH_POD_APPLICATION_NUMBER_SPREADSHEET" xr:uid="{93445971-A6B3-4683-B9ED-4EC2649A5511}"/>
+    <hyperlink ref="H2" location="DEF_WATERSHED_COLUMN_SEARCH_STRING" display="WATERSHED_COLUMN_SEARCH_STRING" xr:uid="{3DA8109F-5025-460F-B94D-26E5003B13CB}"/>
+    <hyperlink ref="I2" location="DEF_SOURCE_NAME_COLUMN_SEARCH_STRING" display="SOURCE_NAME_COLUMN_SEARCH_STRING" xr:uid="{E57F2D8B-2DBA-41E6-BEEC-BC667116A809}"/>
+    <hyperlink ref="J2" location="DEF_TRIB_DESC_COLUMN_SEARCH_STRING" display="TRIB_DESC_COLUMN_SEARCH_STRING" xr:uid="{47538E7D-F5BD-4AF1-8BB9-7E954BEDDC7F}"/>
+    <hyperlink ref="X2" location="DEF_IS_SHAREPOINT_PATH_QAQC_MEASUREMENT_VALUES" display="IS_SHAREPOINT_PATH_QAQC_MEASUREMENT_VALUES" xr:uid="{2796F3B2-5B56-4C81-90CB-623697BE3815}"/>
+    <hyperlink ref="V2" location="DEF_QAQC_MEASUREMENT_VALUES_SPREADSHEET_PATH" display="QAQC_MEASUREMENT_VALUES_SPREADSHEET_PATH" xr:uid="{55003B0F-9F85-4F33-AE2A-F833A902756C}"/>
+    <hyperlink ref="W2" location="DEF_QAQC_MEASUREMENT_VALUES_SPREADSHEET_WORKSHEET_NAME" display="QAQC_MEASUREMENT_VALUES_SPREADSHEET_WORKSHEET_NAME" xr:uid="{A7CF35CA-94DC-43B7-BB79-1A436B41D0F3}"/>
+    <hyperlink ref="AL2" location="DEF_SUBBASIN_POLYGONS_DATABASE_PATH" display="SUBBASIN_POLYGONS_DATABASE_PATH" xr:uid="{C4C102A6-1FBB-4666-8B15-EFA18CA68908}"/>
+    <hyperlink ref="AM2" location="DEF_SUBBASIN_POLYGONS_LAYER_NAME" display="SUBBASIN_POLYGONS_LAYER_NAME" xr:uid="{DC257581-78C3-40E5-B24A-59C01F8231D3}"/>
+    <hyperlink ref="AN2" location="DEF_IS_SHAREPOINT_PATH_SUBBASIN_POLYGONS" display="IS_SHAREPOINT_PATH_SUBBASIN_POLYGONS" xr:uid="{77276DAA-B389-48F1-90C9-2EAD01AAA728}"/>
+    <hyperlink ref="AO2" location="DEF_SUBBASIN_FIELD_ID_NAMES" display="SUBBASIN_FIELD_ID_NAMES" xr:uid="{174AF97C-F07C-4970-BE83-486F3D0014FC}"/>
+    <hyperlink ref="AS2" location="DEF_SUBBASIN_MANUAL_ASSIGNMENT_SPREADSHEET_PATH" display="SUBBASIN_MANUAL_ASSIGNMENT_SPREADSHEET_PATH" xr:uid="{33EBA2E4-0FBA-48C7-8A43-AC6242821539}"/>
+    <hyperlink ref="AT2" location="DEF_SUBBASIN_MANUAL_ASSIGNMENT_WORKSHEET_NAME" display="SUBBASIN_MANUAL_ASSIGNMENT_WORKSHEET_NAME" xr:uid="{0B1DEE05-94E3-4E0D-96D7-B50063C21133}"/>
+    <hyperlink ref="AU2" location="IS_SHAREPOINT_PATH_SUBBASIN_MANUAL_ASSIGNMENT" display="IS_SHAREPOINT_PATH_SUBBASIN_MANUAL_ASSIGNMENT" xr:uid="{A29D92E3-255E-4AE3-AC73-92CCFC7FC661}"/>
+    <hyperlink ref="AE2" location="DEF_NA_REPORTS_SPREADSHEET_PATH" display="NA_REPORTS_SPREADSHEET_PATH" xr:uid="{B995A17C-FCF7-4ED1-933D-00BE31FADD66}"/>
+    <hyperlink ref="AF2" location="DEF_NA_REPORTS_WORKSHEET_NAME" display="NA_REPORTS_WORKSHEET_NAME" xr:uid="{6A6A3F67-2FE2-4B33-9D75-BA533F9A3AB0}"/>
+    <hyperlink ref="AG2" location="DEF_IS_SHAREPOINT_PATH_NA_REPORTS_SPREADSHEET" display="IS_SHAREPOINT_PATH_NA_REPORTS_SPREADSHEET" xr:uid="{95415EA4-6F34-43DC-9BDB-548DF46BD083}"/>
+    <hyperlink ref="AP2" location="DEF_CONNECTIVITY_MATRIX_SPREADSHEET_PATH" display="CONNECTIVITY_MATRIX_SPREADSHEET_PATH" xr:uid="{5E74688E-EA6A-4805-B667-1AAC623445B0}"/>
+    <hyperlink ref="AQ2" location="DEF_CONNECTIVITY_MATRIX_WORKSHEET_NAME" display="CONNECTIVITY_MATRIX_WORKSHEET_NAME" xr:uid="{6E1364E1-9CBE-4981-8009-6EF041C3D455}"/>
+    <hyperlink ref="AR2" location="DEF_IS_SHAREPOINT_PATH_CONNECTIVITY_MATRIX_SPREADSHEET" display="IS_SHAREPOINT_PATH_CONNECTIVITY_MATRIX_SPREADSHEET" xr:uid="{81A63910-7028-4A75-8BDC-211C3A7D77B7}"/>
+    <hyperlink ref="O2" location="Dictionary!A1" display="EWRIMS_REPORTS_FOLDER_PATH" xr:uid="{8A43C4BA-14A9-4A97-B19F-C68BF3096FFB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3774,14 +3844,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B69755CA-4815-49BC-97C9-A62687C98940}">
   <dimension ref="A1:C47"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="76.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="85.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="81.42578125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="76.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="85.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="81.44140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>229</v>
       </c>
@@ -3792,7 +3862,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>6</v>
       </c>
@@ -3803,7 +3873,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>7</v>
       </c>
@@ -3814,7 +3884,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -3825,7 +3895,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>9</v>
       </c>
@@ -3836,7 +3906,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
@@ -3847,7 +3917,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
@@ -3858,7 +3928,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>12</v>
       </c>
@@ -3869,7 +3939,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>13</v>
       </c>
@@ -3880,7 +3950,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>14</v>
       </c>
@@ -3891,7 +3961,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
         <v>15</v>
       </c>
@@ -3902,7 +3972,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>16</v>
       </c>
@@ -3913,7 +3983,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>17</v>
       </c>
@@ -3924,7 +3994,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>18</v>
       </c>
@@ -3935,7 +4005,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="17" t="s">
         <v>19</v>
       </c>
@@ -3946,7 +4016,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>20</v>
       </c>
@@ -3957,7 +4027,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>21</v>
       </c>
@@ -3968,7 +4038,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
@@ -3979,7 +4049,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>23</v>
       </c>
@@ -3990,7 +4060,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>24</v>
       </c>
@@ -4001,7 +4071,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>25</v>
       </c>
@@ -4012,7 +4082,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>26</v>
       </c>
@@ -4023,7 +4093,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>27</v>
       </c>
@@ -4034,7 +4104,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
         <v>28</v>
       </c>
@@ -4045,7 +4115,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>29</v>
       </c>
@@ -4056,7 +4126,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>30</v>
       </c>
@@ -4067,7 +4137,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>31</v>
       </c>
@@ -4078,7 +4148,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
         <v>32</v>
       </c>
@@ -4089,7 +4159,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>33</v>
       </c>
@@ -4100,7 +4170,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>34</v>
       </c>
@@ -4111,7 +4181,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>35</v>
       </c>
@@ -4122,7 +4192,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
         <v>36</v>
       </c>
@@ -4133,7 +4203,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
         <v>37</v>
       </c>
@@ -4144,7 +4214,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>38</v>
       </c>
@@ -4155,7 +4225,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -4166,7 +4236,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>40</v>
       </c>
@@ -4177,7 +4247,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -4188,7 +4258,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38" s="9" t="s">
         <v>42</v>
       </c>
@@ -4199,7 +4269,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="9" t="s">
         <v>43</v>
       </c>
@@ -4210,7 +4280,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>44</v>
       </c>
@@ -4221,7 +4291,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="105" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
         <v>45</v>
       </c>
@@ -4232,7 +4302,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
         <v>46</v>
       </c>
@@ -4243,7 +4313,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
         <v>47</v>
       </c>
@@ -4254,7 +4324,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
         <v>48</v>
       </c>
@@ -4265,7 +4335,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>49</v>
       </c>
@@ -4276,7 +4346,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
         <v>50</v>
       </c>
@@ -4287,7 +4357,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A47" s="7" t="s">
         <v>51</v>
       </c>
@@ -4351,15 +4421,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="b2cf8adb-cf25-47fc-8c92-b53f2a7e7f06">
@@ -4368,6 +4429,15 @@
     <TaxCatchAll xmlns="851dfaa3-aae8-4c03-b90c-7dd4a6526d0d" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4606,14 +4676,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99CBB6A7-3740-4391-8A8B-E146A75EBE0B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B66245A5-6032-43CA-AFD6-6C5801E9C626}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -4626,6 +4688,14 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="851dfaa3-aae8-4c03-b90c-7dd4a6526d0d"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99CBB6A7-3740-4391-8A8B-E146A75EBE0B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Updated Demand scripts to comply with security requirements
</commit_message>
<xml_diff>
--- a/Demand/InputData/Watershed_Demand_Dataset_Paths.xlsx
+++ b/Demand/InputData/Watershed_Demand_Dataset_Paths.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aprashar\Documents\Github\DWRAT_DataScraping\Demand\InputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0730F106-7ADB-4B44-AC33-8DA3E84392C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14E5273E-3D15-4BC9-B0FB-056661624332}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8961FACC-9C35-4F39-BB8E-E3D4A8B78A2C}"/>
   </bookViews>
@@ -121,7 +121,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="174">
   <si>
     <t>Info</t>
   </si>
@@ -294,48 +294,27 @@
     <t>RR</t>
   </si>
   <si>
-    <t>GIS/Russian River.gdb</t>
-  </si>
-  <si>
     <t>RR_NHD_1801_HUC8</t>
   </si>
   <si>
     <t>Russian</t>
   </si>
   <si>
-    <t>SOPs + Documentation\3. Demand Data\SDU Methodology\GIS Steps\RR_pod_points_Merge_filtered_PA_2023-09-19.xlsx</t>
-  </si>
-  <si>
     <t>RR_pod_points_Merge_filtered_PA</t>
   </si>
   <si>
-    <t>SOPs + Documentation\3. Demand Data\SDU Methodology\Non-GIS_Manual_Reviews\RR_Expected_Demand_Units_QAQC.xlsx</t>
-  </si>
-  <si>
     <t>Corrected Data</t>
   </si>
   <si>
-    <t>SOPs + Documentation\3. Demand Data\SDU Methodology\Non-GIS_Manual_Reviews\RR_Expected_Demand_Units_QAQC_Measurement_Values.xlsx</t>
-  </si>
-  <si>
     <t>Data</t>
   </si>
   <si>
-    <t>SOPs + Documentation\3. Demand Data\SDU Methodology\Non-GIS_Manual_Reviews\RR_Expected_Demand_Units_QAQC_Median_Based.xlsx</t>
-  </si>
-  <si>
     <t>Filtered Data</t>
   </si>
   <si>
-    <t>SOPs + Documentation\3. Demand Data\SDU Methodology\Non-GIS_Manual_Reviews\RR_Duplicate_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
     <t>Sheet1</t>
   </si>
   <si>
-    <t>SOPs + Documentation\3. Demand Data\SDU Methodology\Non-GIS_Manual_Reviews\RR_Empty_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
     <t>NAD83</t>
   </si>
   <si>
@@ -348,9 +327,6 @@
     <t>Basin_ID; Basin_Num; Grouping</t>
   </si>
   <si>
-    <t>SOPs + Documentation\3. Demand Data\SDU Methodology\GIS Steps\RR_Missing_MainStem_GIS_Manual_Assignment.xlsx</t>
-  </si>
-  <si>
     <t>Missing_MainStem_GIS</t>
   </si>
   <si>
@@ -360,454 +336,16 @@
     <t>NV</t>
   </si>
   <si>
-    <t>Program Watersheds/1. Watershed Folders/Navarro River/Data/GIS Datasets/Navarro_River_Watershed_GIS/Navarro_River_Watershed.gpkg</t>
-  </si>
-  <si>
     <t>WBD_HU10_Navarro</t>
   </si>
   <si>
     <t>Navarro</t>
   </si>
   <si>
-    <t>Program Watersheds/1. Watershed Folders/Navarro River/Data/GIS Preprocessing/NV_GIS_Preprocessing.xlsx</t>
-  </si>
-  <si>
     <t>R_Review</t>
   </si>
   <si>
-    <t>Program Watersheds\1. Watershed Folders\Navarro River\Data\GIS Preprocessing\Reports</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Navarro River/Data/GIS Preprocessing/NV_POD_StreamStats_Review.xlsx</t>
-  </si>
-  <si>
     <t>Final_List</t>
-  </si>
-  <si>
-    <t>Program Watersheds/1. Watershed Folders/Navarro River/Data/Demand QAQC/NV_Expected_Demand_Units_QAQC.xlsx</t>
-  </si>
-  <si>
-    <t>Sheet 1</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Navarro River/Data/Demand QAQC/NV_Expected_Demand_Units_QAQC_Median_Based.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders/Navarro River/Data/Demand QAQC/NV_Duplicate_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders/Navarro River/Data/Demand QAQC/NV_Empty_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders/Navarro River/Data/GIS Preprocessing/NV_POD_StreamStats_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders/Navarro River/Data/GIS Datasets/NHDPlus_Delineations/LSPC_Delineations</t>
-  </si>
-  <si>
-    <t>NHDPlusCatchment_EditedforLSPC</t>
-  </si>
-  <si>
-    <t>FEATUREID; FromNode; ToNode; ReachCode</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders/Navarro River/Data/GIS Datasets/NHDPlus_Delineations/LSPC_Delineations/UpstreamNetwork_Matrix.xlsx</t>
-  </si>
-  <si>
-    <t>LSPC_Matrix</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders/Navarro River/Data/Demand QAQC/NV_POD_Subbasin_Assignment.xlsx</t>
-  </si>
-  <si>
-    <t>Review</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Navarro River\Data\Demand QAQC\NV_POD_Subbasin_Assignment.xlsx</t>
-  </si>
-  <si>
-    <t>Napa River</t>
-  </si>
-  <si>
-    <t>NR</t>
-  </si>
-  <si>
-    <t>Program Watersheds/1. Watershed Folders/Napa River/Data/GIS/Demand Analysis (1.26.23)/NapaRive_PreProcessing.gdb</t>
-  </si>
-  <si>
-    <t>Napa</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Napa River\Data\GIS\Demand Analysis (1.26.23)\NR_pod_points_filtered_042924.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Napa River\Data\Manual Review\NR_Expected_Demand_Units_QAQC.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Napa River\Data\Manual Review\NR_Expected_Demand_Units_QAQC_Median_Based.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Napa River\Data\Manual Review\NR_Duplicate_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Napa River\Data\Manual Review\NR_Empty_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Napa River\Deliverables\Model Dev Report\Napa_LSPC_Delineations</t>
-  </si>
-  <si>
-    <t>NHDPlusCatchmentHR_EditedforLSPC</t>
-  </si>
-  <si>
-    <t>New_SWSID; NHDPlusID</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Napa River\Deliverables\Model Dev Report\Napa_LSPC_Delineations\UpstreamNetwork_Matrix_Napa_newIDs.xlsx</t>
-  </si>
-  <si>
-    <t>ConMat</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>Butte Creek</t>
-  </si>
-  <si>
-    <t>BC</t>
-  </si>
-  <si>
-    <t>Program Watersheds/1. Watershed Folders/Butte Creek/Data/GIS/BC_Demand.gdb</t>
-  </si>
-  <si>
-    <t>BC_NHD_HUC8</t>
-  </si>
-  <si>
-    <t>Butte</t>
-  </si>
-  <si>
-    <t>Program Watersheds/1. Watershed Folders/Butte Creek/Data/Demand/BC_GIS_Preprocessing_2023-02-26.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Butte Creek\Data\Demand\BC_POD_ ID_List.xlsx</t>
-  </si>
-  <si>
-    <t>Sheet4</t>
-  </si>
-  <si>
-    <t>Program Watersheds/1. Watershed Folders/Butte Creek/Data/Demand/BC_Expected_Demand_Units_QAQC.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds/1. Watershed Folders/Butte Creek/Data/Demand/BC_Expected_Demand_Units_QAQC_Median_Based.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders/Butte Creek/Data/Demand/BC_Duplicate_Reports_Manual_Review2.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Butte Creek\Data\GIS\Final_NHDPlusCatchmentsFlowlines_Sent to Board</t>
-  </si>
-  <si>
-    <t>Butte_Catchments_Final</t>
-  </si>
-  <si>
-    <t>CatchID</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Butte Creek\Data\GIS\Final_NHDPlusCatchmentsFlowlines_Sent to Board\UpstreamNetwork_Butte_Catch.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Butte Creek\Data\Demand\BC_POD_Subbasin_Assignment.xlsx</t>
-  </si>
-  <si>
-    <t>Test Navarro</t>
-  </si>
-  <si>
-    <t>TEST</t>
-  </si>
-  <si>
-    <t>Program Watersheds/1. Watershed Folders\Test Creek\Test_GIS_Preprocessing.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Test Creek\Test_POD_StreamStats_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Test Creek\Manual_Reviews\TEST_Expected_Demand_Units_QAQC.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Test Creek\Manual_Reviews\TEST_Expected_Demand_Units_QAQC_Median_Based.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Test Creek\Manual_Reviews\TEST_Duplicate_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Test Creek\Manual_Reviews\TEST_Empty_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Gualala River</t>
-  </si>
-  <si>
-    <t>GL</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Gualala River\Data\GIS\HUC10</t>
-  </si>
-  <si>
-    <t>Gualala_HUC10_Boundary_</t>
-  </si>
-  <si>
-    <t>Gualala</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Gualala River\Data\GIS_Preprocessing\GL_GIS_Preprocessing.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Gualala River\Data\GIS_Preprocessing\Reports</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Gualala River\Data\GIS_Preprocessing\GL_POD_StreamStats_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Gualala River\Data\Manual_Reviews\GL_Expected_Demand_Units_QAQC.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Gualala River\Data\Manual_Reviews\GL_Expected_Demand_Units_QAQC_Median_Based.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Gualala River\Data\Manual_Reviews\GL_Duplicate_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Gualala River\Data\Manual_Reviews\GL_Empty_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Gualala River\Data\GIS\Delineations\Gualala_Catchments</t>
-  </si>
-  <si>
-    <t>Gualala_Catchments</t>
-  </si>
-  <si>
-    <t>COMID; ToNode; FromNode; OUTBASIN</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Gualala River\Data\GIS\Delineations\Gualala_UpstreamNetworkTable.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Gualala River\Data\GIS_Preprocessing\GL_POD_Subbasin_Assignment.xlsx</t>
-  </si>
-  <si>
-    <t>Salmon Creek</t>
-  </si>
-  <si>
-    <t>SC</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Salmon Creek\Data\GIS\SC_Demand.gdb</t>
-  </si>
-  <si>
-    <t>SC_NHD_HUC12</t>
-  </si>
-  <si>
-    <t>asdfghjkl</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Salmon Creek\Data\GIS Preprocessing\SC_GIS_Preprocessing.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Salmon Creek\Data\GIS Preprocessing\Reports</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Salmon Creek\Data\Demand\Salmon_Final_POD.xlsx</t>
-  </si>
-  <si>
-    <t>POD</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Salmon Creek\Data\Demand\SC_Expected_Demand_Units_QAQC.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Salmon Creek\Data\Demand\SC_Expected_Demand_Units_QAQC_Median_Based.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Salmon Creek\Data\Demand\SC_Duplicate_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>POD_List</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Salmon Creek\Data\GIS\Task 3.1 Delineation\Catchments_EditedforLSPC</t>
-  </si>
-  <si>
-    <t>Catchments_EditedforLSPC</t>
-  </si>
-  <si>
-    <t>COMID; ToNode; FromNode; OutBasin</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Salmon Creek\Data\GIS\Task 3.1 Delineation\Salmon_UpstreamNetworkTable.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Salmon Creek\Data\Demand\SC_POD_Subbasin_Assignment.xlsx</t>
-  </si>
-  <si>
-    <t>Tomales-Drake Bays</t>
-  </si>
-  <si>
-    <t>TD</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Tomales-Drake Bays\Data\GIS\HUC8</t>
-  </si>
-  <si>
-    <t>TomalesDrakeBays_HUC8_Boundary_</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Tomales-Drake Bays\Data\GIS_Preprocessing\TD_GIS_Preprocessing.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Tomales-Drake Bays\Data\TDB_ReviewedPODs.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Tomales-Drake Bays\Data\Manual Reviews\TD_Expected_Demand_Units_QAQC.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Tomales-Drake Bays\Data\Manual Reviews\TD_Expected_Demand_Units_QAQC_Median_Based.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Tomales-Drake Bays\Data\Manual Reviews\TD_Duplicate_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Tomales-Drake Bays\Data\Manual Reviews\TD_Empty_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Tomales-Drake Bays\Data\Paradigm-Sourced\TomalesDrake_Catchments</t>
-  </si>
-  <si>
-    <t>TomalesDrake_Catchments</t>
-  </si>
-  <si>
-    <t>COMID;FromNode;ToNode</t>
-  </si>
-  <si>
-    <t>Test Russian</t>
-  </si>
-  <si>
-    <t>TR</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Test Watersheds\Test_Russian\Data\GIS_Preprocessing\TR_GIS_Preprocessing_2025-03-17.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Test_Russian\Data\GIS_Preprocessing\Reports</t>
-  </si>
-  <si>
-    <t>Final_POD_List</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Test Watersheds\Test_Russian\Data\Demand_QAQC\TR_Expected_Demand_Units_QAQC_SharePoint.xlsx</t>
-  </si>
-  <si>
-    <t>Main_Table</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Test Watersheds\Test_Russian\Data\Demand_QAQC\RR_Expected_Demand_Units_QAQC_Measurement_Values.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Test Watersheds\Test_Russian\Data\Demand_QAQC\TR_Expected_Demand_Units_QAQC_Median_Based_SharePoint.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Test Watersheds\Test_Russian\Data\Demand_QAQC\TR_Duplicate_Reports_Manual_Review_SharePoint.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Test Watersheds\Test_Russian\Data\Demand_QAQC\TR_Empty_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Test Watersheds\Test_Russian\Data\Demand_QAQC\TR_POD_Subbasin_Assignment.xlsx</t>
-  </si>
-  <si>
-    <t>South Fork Trinity</t>
-  </si>
-  <si>
-    <t>SFT</t>
-  </si>
-  <si>
-    <t>SFT_HUC8</t>
-  </si>
-  <si>
-    <t>SouthForkTrinity</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\South Fork Trinity\Data\GIS_Preprocessing\Reports</t>
-  </si>
-  <si>
-    <t>Mattole River</t>
-  </si>
-  <si>
-    <t>MT</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Mattole River\Data\GIS\HUC8</t>
-  </si>
-  <si>
-    <t>Mattole_HUC8_Boundary_</t>
-  </si>
-  <si>
-    <t>Mattole</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Mattole River\Data\GIS_Preprocessing\MT_GIS_Preprocessing.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Mattole River\Data\GIS_Preprocessing\Reports</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Putah Creek </t>
-  </si>
-  <si>
-    <t xml:space="preserve">PC </t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Putah Creek\Data\GIS\HUC8</t>
-  </si>
-  <si>
-    <t>UpperPutah_HUC8_Boundary_</t>
-  </si>
-  <si>
-    <t>Putah Creek</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Putah Creek\Data\GIS_Preprocessing\Putah Creek Watershed_PODs.xlsx</t>
-  </si>
-  <si>
-    <t>Final</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Putah Creek\Data\Manual Review\PC_Expected_Demand_Units_QAQC.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Putah Creek\Data\Manual Review\PC_Expected_Demand_Units_QAQC_Median_Based.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Putah Creek\Data\Manual Review\PC_Duplicate_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Putah Creek\Data\Manual Review\PC_Empty_Reports_Manual_Review.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Putah Creek\Deliverables\Watershed Delineations\Catchments_EditedforLSPC</t>
-  </si>
-  <si>
-    <t>Putah_Catchments_EditedforLSPC</t>
-  </si>
-  <si>
-    <t>COMID; FromNode; ToNode</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Putah Creek\Deliverables\Watershed Delineations\Putah_UpstreamNetworkTable.csv</t>
-  </si>
-  <si>
-    <t>Putah_UpstreamNetworkTable</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Putah Creek\Data\Manual Review\PC_POD_Subbasin_Assignment.xlsx</t>
   </si>
   <si>
     <t>COLUMN_NAME</t>
@@ -939,9 +477,6 @@
     <t>The index number of the R variable "wsPoint" that corresponds to the exit point of the watershed boundary</t>
   </si>
   <si>
-    <t>Required for "POD_StreamStats_Analysis.R". The script uses a single point to represent the exit location of the watershed's main tributary. The watershed boundary layer is required to identify this exit point. For more details, see Step 4e of "Updating the Demand Data Scripts.docx" (click on this cell to go there).</t>
-  </si>
-  <si>
     <t>Path to the manually reviewed GIS Pre-Processing spreadsheet</t>
   </si>
   <si>
@@ -1126,79 +661,52 @@
     <t>Is "SUBBASIN_MANUAL_ASSIGNMENT_SPREADSHEET_PATH" a SharePoint path?</t>
   </si>
   <si>
-    <t>Program Watersheds\1. Watershed Folders\Tomales-Drake Bays\Data\Paradigm-Sourced\TomalesDrake_UpstreamNetworkTable.xlsx</t>
-  </si>
-  <si>
-    <t>TomalesDrake_UpstreamNetworkTab</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Tomales-Drake Bays\Data\TD_POD_Subbasin_Assignment.xlsx</t>
-  </si>
-  <si>
-    <t>Pre_Filtered</t>
-  </si>
-  <si>
-    <t>Final_List_Paradigm</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Trinity River\Data\POD_Mannual Review\SFT_POD_Coordinates.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Trinity River\Data\GIS\HUC8</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Trinity River\Data\POD_Mannual Review\SFT_GIS_Preprocessing.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Mattole River\Data\Demand_QAQC\MT_Expected_Demand_Units_QAQC_SharePoint.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Mattole River\Data\Demand_QAQC\MT_Expected_Demand_Units_QAQC_Median_Based_SharePoint.xlsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Program Watersheds\1. Watershed Folders\Mattole River\Data\Demand_QAQC\MT_Duplicate_Reports_Manual_Review_SharePoint.xlsx</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Mattole River\Data\GIS\Catchments_EditedforLSPC</t>
-  </si>
-  <si>
-    <t>COMID</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Mattole River\Data\GIS\Mattole_UpstreamNetworkTable.xlsx</t>
-  </si>
-  <si>
-    <t>Table1</t>
-  </si>
-  <si>
-    <t>Program Watersheds\1. Watershed Folders\Mattole River\Data\Demand_QAQC\MT_POD_Subbasin_Assignment.xlsx</t>
-  </si>
-  <si>
-    <t>NR__WB</t>
-  </si>
-  <si>
-    <t>TestMattole River</t>
-  </si>
-  <si>
-    <t>TEST_MT</t>
-  </si>
-  <si>
-    <t>C:\Users\amoussalli\Downloads\Mattole_HUC8\HUC8</t>
-  </si>
-  <si>
-    <t>Delta</t>
-  </si>
-  <si>
-    <t>DL</t>
-  </si>
-  <si>
-    <t>C:\Users\aprashar\Documents\Github\DWRAT_DataScraping\Demand\InputData\i03_LegalDeltaBoundary.geojson</t>
-  </si>
-  <si>
     <t>EXCLUDED_REPORTING_YEARS</t>
   </si>
   <si>
     <t>2021;2022</t>
+  </si>
+  <si>
+    <t>EXAMPLE/Russian River.gdb</t>
+  </si>
+  <si>
+    <t>InputData/Navarro_River_Watershed.gpkg</t>
+  </si>
+  <si>
+    <t>OutputData/NV_GIS_Preprocessing.xlsx</t>
+  </si>
+  <si>
+    <t>InputData/Reports</t>
+  </si>
+  <si>
+    <t>RR_pod_points_Merge_filtered_PA_2023-09-19.xlsx</t>
+  </si>
+  <si>
+    <t>Example_Path\NV_POD_StreamStats_Review.xlsx</t>
+  </si>
+  <si>
+    <t>Sheet_1</t>
+  </si>
+  <si>
+    <t>RR_Expected_Demand_Units_QAQC.xlsx</t>
+  </si>
+  <si>
+    <t>RR_Expected_Demand_Units_QAQC_Measurement_Values.xlsx</t>
+  </si>
+  <si>
+    <t>RR_Expected_Demand_Units_QAQC_Median_Based.xlsx</t>
+  </si>
+  <si>
+    <t>RR_Duplicate_Reports_Manual_Review.xlsx</t>
+  </si>
+  <si>
+    <t>RR_Empty_Reports_Manual_Review.xlsx</t>
+  </si>
+  <si>
+    <t>RR_Missing_MainStem_GIS_Manual_Assignment.xlsx</t>
+  </si>
+  <si>
+    <t>Required for "POD_StreamStats_Analysis.R". The script uses a single point to represent the exit location of the watershed's main tributary. The watershed boundary layer is required to identify this exit point. (Please consult the documentation for more information)</t>
   </si>
 </sst>
 </file>
@@ -1386,6 +894,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1399,12 +913,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1440,18 +948,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="23">
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thick">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1567,6 +1063,18 @@
       </border>
     </dxf>
     <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thick">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -1614,21 +1122,21 @@
     </tableColumn>
     <tableColumn id="2" xr3:uid="{D398884F-42D5-47C1-B3FC-B226E40F56C9}" name="NAME"/>
     <tableColumn id="3" xr3:uid="{4FACAB44-BBA1-4B8A-BF3E-060B26921A3E}" name="ID" dataDxfId="20"/>
-    <tableColumn id="51" xr3:uid="{B7595ECA-A15A-4155-8B15-4800F18CCDFD}" name="EXCLUDED_REPORTING_YEARS" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{321EF454-3BDA-4FED-84A0-242C6CFD30CE}" name="WATERSHED_BOUNDARY_DATABASE_PATH" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{18A10455-06B2-4B6E-9D24-48D247873D5B}" name="WATERSHED_BOUNDARY_LAYER_NAME" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{A44DDF5D-002A-45F2-87CD-E4BDCC91F051}" name="IS_SHAREPOINT_PATH_WATERSHED_BOUNDARY" dataDxfId="17"/>
-    <tableColumn id="26" xr3:uid="{A34CFBB5-3CA3-471B-8C9D-FFD2620BEE67}" name="WATERSHED_COLUMN_SEARCH_STRING" dataDxfId="16"/>
-    <tableColumn id="27" xr3:uid="{B752EE02-609B-45A5-9A8B-B23ECE55E9DF}" name="SOURCE_NAME_COLUMN_SEARCH_STRING" dataDxfId="15"/>
-    <tableColumn id="28" xr3:uid="{6784E5FE-7D00-4755-B3D1-7E214D9D6EFA}" name="TRIB_DESC_COLUMN_SEARCH_STRING" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{1AF87C52-D944-4D7B-A074-D3ED32FFAA03}" name="WATERSHED_EXIT_POINT_INDEX" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{AC0EB44C-3D57-4B3D-B2AA-2B91C7692534}" name="GIS_PREPROCESSING_SPREADSHEET_PATH" dataDxfId="12"/>
+    <tableColumn id="51" xr3:uid="{B7595ECA-A15A-4155-8B15-4800F18CCDFD}" name="EXCLUDED_REPORTING_YEARS" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{321EF454-3BDA-4FED-84A0-242C6CFD30CE}" name="WATERSHED_BOUNDARY_DATABASE_PATH" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{18A10455-06B2-4B6E-9D24-48D247873D5B}" name="WATERSHED_BOUNDARY_LAYER_NAME" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{A44DDF5D-002A-45F2-87CD-E4BDCC91F051}" name="IS_SHAREPOINT_PATH_WATERSHED_BOUNDARY" dataDxfId="16"/>
+    <tableColumn id="26" xr3:uid="{A34CFBB5-3CA3-471B-8C9D-FFD2620BEE67}" name="WATERSHED_COLUMN_SEARCH_STRING" dataDxfId="15"/>
+    <tableColumn id="27" xr3:uid="{B752EE02-609B-45A5-9A8B-B23ECE55E9DF}" name="SOURCE_NAME_COLUMN_SEARCH_STRING" dataDxfId="14"/>
+    <tableColumn id="28" xr3:uid="{6784E5FE-7D00-4755-B3D1-7E214D9D6EFA}" name="TRIB_DESC_COLUMN_SEARCH_STRING" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{1AF87C52-D944-4D7B-A074-D3ED32FFAA03}" name="WATERSHED_EXIT_POINT_INDEX" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{AC0EB44C-3D57-4B3D-B2AA-2B91C7692534}" name="GIS_PREPROCESSING_SPREADSHEET_PATH" dataDxfId="11"/>
     <tableColumn id="9" xr3:uid="{B00750ED-07CA-4479-AFF3-3151E1E0F833}" name="GIS_PREPROCESSING_WORKSHEET_NAME"/>
-    <tableColumn id="10" xr3:uid="{812E332A-6EEB-4CA3-A2D6-4547CD7C54A4}" name="IS_SHAREPOINT_PATH_GIS_PREPROCESSING_SPREADSHEET" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{812E332A-6EEB-4CA3-A2D6-4547CD7C54A4}" name="IS_SHAREPOINT_PATH_GIS_PREPROCESSING_SPREADSHEET" dataDxfId="10"/>
     <tableColumn id="46" xr3:uid="{49AF8B55-F40C-42E4-A524-B49C4F8CF00A}" name="EWRIMS_REPORTS_FOLDER_PATH"/>
     <tableColumn id="29" xr3:uid="{D03F612F-DD50-4A34-9AC0-CD6674450BE6}" name="POD_APPLICATION_NUMBER_SPREADSHEET_PATH"/>
     <tableColumn id="30" xr3:uid="{C2AD24F7-0584-49C9-A672-C8DD7146A417}" name="POD_APPLICATION_NUMBER_WORKSHEET_NAME"/>
-    <tableColumn id="31" xr3:uid="{66CE7497-E596-413F-8921-544BB74C3DD7}" name="IS_SHAREPOINT_PATH_POD_APPLICATION_NUMBER_SPREADSHEET" dataDxfId="10"/>
+    <tableColumn id="31" xr3:uid="{66CE7497-E596-413F-8921-544BB74C3DD7}" name="IS_SHAREPOINT_PATH_POD_APPLICATION_NUMBER_SPREADSHEET" dataDxfId="9"/>
     <tableColumn id="11" xr3:uid="{5DB7ED87-871F-4C06-8BF4-35668661F916}" name="QAQC_UNIT_CONVERSION_ERRORS_SPREADSHEET_PATH"/>
     <tableColumn id="12" xr3:uid="{3442F1AA-5583-49F9-916A-1D3BE29BF0E0}" name="QAQC_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME"/>
     <tableColumn id="13" xr3:uid="{DCBCDD9C-561B-45B9-A277-8DC826228F9D}" name="IS_SHAREPOINT_PATH_QAQC_UNIT_CONVERSION_ERRORS_SPREADSHEET"/>
@@ -1636,21 +1144,21 @@
     <tableColumn id="24" xr3:uid="{4402E847-8344-4AC0-83BD-027C2C85F955}" name="QAQC_MEASUREMENT_VALUES_SPREADSHEET_WORKSHEET_NAME"/>
     <tableColumn id="23" xr3:uid="{BF3DBB2A-B4D9-497B-9AA9-202689EB04F8}" name="IS_SHAREPOINT_PATH_QAQC_MEASUREMENT_VALUES"/>
     <tableColumn id="14" xr3:uid="{1F6934E6-F4A1-4438-909C-60C56721DB48}" name="QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET_PATH"/>
-    <tableColumn id="15" xr3:uid="{B0C47A36-9A34-4BBF-8403-827FA51FD727}" name="QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME" dataDxfId="9"/>
-    <tableColumn id="16" xr3:uid="{538377CD-C686-44C6-87ED-6ABD5DF88F83}" name="IS_SHAREPOINT_PATH_QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET" dataDxfId="8"/>
-    <tableColumn id="17" xr3:uid="{C9FB89DE-1AD6-4FEC-8961-82B10F599F29}" name="QAQC_DUPLICATE_REPORTING_SPREADSHEET_PATH" dataDxfId="7"/>
-    <tableColumn id="18" xr3:uid="{0E0BCAD4-6245-49D8-AE35-419FAD1FA06B}" name="QAQC_DUPLICATE_REPORTING_WORKSHEET_NAME" dataDxfId="6"/>
-    <tableColumn id="19" xr3:uid="{5AF9174D-850A-401C-8553-F941816CB39D}" name="IS_SHAREPOINT_PATH_QAQC_DUPLICATE_REPORTING_SPREADSHEET" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{B0C47A36-9A34-4BBF-8403-827FA51FD727}" name="QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_WORKSHEET_NAME" dataDxfId="8"/>
+    <tableColumn id="16" xr3:uid="{538377CD-C686-44C6-87ED-6ABD5DF88F83}" name="IS_SHAREPOINT_PATH_QAQC_MEDIAN_BASED_UNIT_CONVERSION_ERRORS_SPREADSHEET" dataDxfId="7"/>
+    <tableColumn id="17" xr3:uid="{C9FB89DE-1AD6-4FEC-8961-82B10F599F29}" name="QAQC_DUPLICATE_REPORTING_SPREADSHEET_PATH" dataDxfId="6"/>
+    <tableColumn id="18" xr3:uid="{0E0BCAD4-6245-49D8-AE35-419FAD1FA06B}" name="QAQC_DUPLICATE_REPORTING_WORKSHEET_NAME" dataDxfId="5"/>
+    <tableColumn id="19" xr3:uid="{5AF9174D-850A-401C-8553-F941816CB39D}" name="IS_SHAREPOINT_PATH_QAQC_DUPLICATE_REPORTING_SPREADSHEET" dataDxfId="4"/>
     <tableColumn id="42" xr3:uid="{2E400177-88F2-41C0-8BDB-5818D102917B}" name="NA_REPORTS_SPREADSHEET_PATH"/>
     <tableColumn id="41" xr3:uid="{3CD8CF08-7BC6-467E-8C6D-253F1DFF6541}" name="NA_REPORTS_WORKSHEET_NAME"/>
-    <tableColumn id="40" xr3:uid="{8AC94F1A-65B4-4A42-AA0D-212073E77362}" name="IS_SHAREPOINT_PATH_NA_REPORTS_SPREADSHEET" dataDxfId="4"/>
+    <tableColumn id="40" xr3:uid="{8AC94F1A-65B4-4A42-AA0D-212073E77362}" name="IS_SHAREPOINT_PATH_NA_REPORTS_SPREADSHEET" dataDxfId="3"/>
     <tableColumn id="32" xr3:uid="{281E90F9-0915-4C7E-B4B0-D3A865435D1A}" name="POD_COORDINATES_SPREADSHEET_PATH"/>
     <tableColumn id="33" xr3:uid="{11DF8B48-852D-46FB-8541-B4DBAB7A1AB6}" name="POD_COORDINATES_WORKSHEET_NAME"/>
     <tableColumn id="35" xr3:uid="{FE79FDB1-2CE3-42C6-90E4-3857101E5E8A}" name="IS_SHAREPOINT_PATH_POD_COORDINATES_SPREADSHEET"/>
     <tableColumn id="34" xr3:uid="{47BF0670-01C9-478D-9F45-481314955B4E}" name="POD_COORDINATES_REFERENCE_SYSTEM"/>
     <tableColumn id="20" xr3:uid="{6557FF05-7172-4057-9259-C83EA504646F}" name="SUBBASIN_POLYGONS_DATABASE_PATH"/>
     <tableColumn id="21" xr3:uid="{71DF2163-A7B7-471B-909E-7C0B1372B75B}" name="SUBBASIN_POLYGONS_LAYER_NAME"/>
-    <tableColumn id="22" xr3:uid="{4731AD94-4A54-4E5D-8226-C553D6203196}" name="IS_SHAREPOINT_PATH_SUBBASIN_POLYGONS" dataDxfId="3"/>
+    <tableColumn id="22" xr3:uid="{4731AD94-4A54-4E5D-8226-C553D6203196}" name="IS_SHAREPOINT_PATH_SUBBASIN_POLYGONS" dataDxfId="2"/>
     <tableColumn id="36" xr3:uid="{79EB03EB-27F7-40E3-B85F-9A85C71A18D9}" name="SUBBASIN_FIELD_ID_NAMES"/>
     <tableColumn id="45" xr3:uid="{1FF3574F-AF8C-465E-B27F-34F613EB9725}" name="CONNECTIVITY_MATRIX_SPREADSHEET_PATH"/>
     <tableColumn id="44" xr3:uid="{F6CF9B50-BFEF-4799-8DBA-489BED7B2892}" name="CONNECTIVITY_MATRIX_WORKSHEET_NAME"/>
@@ -1670,9 +1178,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{14D3AF92-57CC-48E0-916C-527CCD353E2B}" name="Table4" displayName="Table4" ref="A1:C47" totalsRowShown="0">
   <autoFilter ref="A1:C47" xr:uid="{14D3AF92-57CC-48E0-916C-527CCD353E2B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{47B19E1B-043A-4C10-A456-3179E3432197}" name="COLUMN_NAME" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{47B19E1B-043A-4C10-A456-3179E3432197}" name="COLUMN_NAME" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{7C95D3E6-5AC8-446C-AA32-9C6FCCE24F43}" name="DEFINITION"/>
-    <tableColumn id="3" xr3:uid="{4D580C7B-D92C-44C5-BD46-100E46839D1B}" name="DESCRIPTION" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{4D580C7B-D92C-44C5-BD46-100E46839D1B}" name="DESCRIPTION" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2048,24 +1556,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="25" t="s">
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="27"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="29"/>
       <c r="O1" s="22"/>
       <c r="P1" s="33" t="s">
         <v>2</v>
@@ -2091,25 +1599,25 @@
       </c>
       <c r="AF1" s="37"/>
       <c r="AG1" s="38"/>
-      <c r="AH1" s="23" t="s">
+      <c r="AH1" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="AI1" s="24"/>
-      <c r="AJ1" s="24"/>
-      <c r="AK1" s="24"/>
-      <c r="AL1" s="24"/>
-      <c r="AM1" s="24"/>
-      <c r="AN1" s="24"/>
-      <c r="AO1" s="24"/>
-      <c r="AP1" s="24"/>
-      <c r="AQ1" s="24"/>
-      <c r="AR1" s="24"/>
-      <c r="AS1" s="24"/>
-      <c r="AT1" s="24"/>
-      <c r="AU1" s="24"/>
-      <c r="AV1" s="24"/>
-      <c r="AW1" s="24"/>
-      <c r="AX1" s="24"/>
+      <c r="AI1" s="26"/>
+      <c r="AJ1" s="26"/>
+      <c r="AK1" s="26"/>
+      <c r="AL1" s="26"/>
+      <c r="AM1" s="26"/>
+      <c r="AN1" s="26"/>
+      <c r="AO1" s="26"/>
+      <c r="AP1" s="26"/>
+      <c r="AQ1" s="26"/>
+      <c r="AR1" s="26"/>
+      <c r="AS1" s="26"/>
+      <c r="AT1" s="26"/>
+      <c r="AU1" s="26"/>
+      <c r="AV1" s="26"/>
+      <c r="AW1" s="26"/>
+      <c r="AX1" s="26"/>
     </row>
     <row r="2" spans="1:50" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
@@ -2122,7 +1630,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>336</v>
+        <v>158</v>
       </c>
       <c r="E2" s="13" t="s">
         <v>9</v>
@@ -2265,7 +1773,7 @@
     </row>
     <row r="3" spans="1:50" s="11" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="11">
-        <f t="shared" ref="A3:A6" si="0">ROW(B3) - 2</f>
+        <f t="shared" ref="A3:A4" si="0">ROW(B3) - 2</f>
         <v>1</v>
       </c>
       <c r="B3" s="11" t="s">
@@ -2275,25 +1783,25 @@
         <v>56</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>337</v>
+        <v>159</v>
       </c>
       <c r="E3" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="F3" s="12" t="s">
         <v>57</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>58</v>
       </c>
       <c r="G3" s="12" t="b">
         <v>1</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J3" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K3" s="20">
         <v>6672</v>
@@ -2301,88 +1809,88 @@
       <c r="L3" s="12"/>
       <c r="N3" s="10"/>
       <c r="P3" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="Q3" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="R3" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="S3" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="T3" s="11" t="s">
         <v>60</v>
-      </c>
-      <c r="Q3" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="R3" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="S3" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="T3" s="11" t="s">
-        <v>63</v>
       </c>
       <c r="U3" s="11" t="b">
         <v>1</v>
       </c>
       <c r="V3" s="11" t="s">
-        <v>64</v>
+        <v>168</v>
       </c>
       <c r="W3" s="11" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="X3" s="11" t="b">
         <v>1</v>
       </c>
       <c r="Y3" s="11" t="s">
-        <v>66</v>
+        <v>169</v>
       </c>
       <c r="Z3" s="12" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="AA3" s="12" t="b">
         <v>1</v>
       </c>
       <c r="AB3" s="12" t="s">
-        <v>68</v>
+        <v>170</v>
       </c>
       <c r="AC3" s="12" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="AD3" s="10" t="b">
         <v>1</v>
       </c>
       <c r="AE3" s="11" t="s">
-        <v>70</v>
+        <v>171</v>
       </c>
       <c r="AF3" s="11" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="AG3" s="11" t="b">
         <v>1</v>
       </c>
       <c r="AH3" s="11" t="s">
-        <v>60</v>
+        <v>164</v>
       </c>
       <c r="AI3" s="11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="AJ3" s="11" t="b">
         <v>1</v>
       </c>
       <c r="AK3" s="11" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="AL3" s="11" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="AM3" s="11" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="AN3" s="11" t="b">
         <v>0</v>
       </c>
       <c r="AO3" s="11" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="AS3" s="11" t="s">
-        <v>75</v>
+        <v>172</v>
       </c>
       <c r="AT3" s="11" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="AU3" s="11" t="b">
         <v>1</v>
@@ -2394,1386 +1902,180 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="2" t="s">
-        <v>79</v>
+        <v>161</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="G4" s="12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="K4" s="15">
         <v>525</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>82</v>
+        <v>162</v>
       </c>
       <c r="M4" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="N4" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O4" t="s">
-        <v>84</v>
+        <v>163</v>
       </c>
       <c r="P4" t="s">
-        <v>85</v>
+        <v>165</v>
       </c>
       <c r="Q4" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="R4" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="S4" t="s">
-        <v>87</v>
-      </c>
-      <c r="T4" t="s">
-        <v>88</v>
-      </c>
-      <c r="U4" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>89</v>
-      </c>
-      <c r="Z4" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB4" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="AC4" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AD4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE4" t="s">
-        <v>91</v>
-      </c>
-      <c r="AF4" t="s">
-        <v>69</v>
-      </c>
-      <c r="AG4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH4" t="s">
-        <v>92</v>
-      </c>
-      <c r="AI4" t="s">
-        <v>86</v>
-      </c>
-      <c r="AJ4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK4" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL4" t="s">
-        <v>93</v>
-      </c>
-      <c r="AM4" t="s">
-        <v>94</v>
-      </c>
-      <c r="AN4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AO4" t="s">
-        <v>95</v>
-      </c>
-      <c r="AP4" t="s">
-        <v>96</v>
-      </c>
-      <c r="AQ4" t="s">
-        <v>97</v>
-      </c>
-      <c r="AR4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AS4" t="s">
-        <v>98</v>
-      </c>
-      <c r="AT4" t="s">
-        <v>99</v>
-      </c>
-      <c r="AU4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AV4" t="s">
-        <v>100</v>
-      </c>
-      <c r="AW4" t="s">
-        <v>69</v>
-      </c>
-      <c r="AX4" t="b">
-        <v>1</v>
-      </c>
+      <c r="AD4" s="1"/>
     </row>
     <row r="5" spans="1:50" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>101</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>102</v>
-      </c>
+      <c r="C5" s="1"/>
       <c r="D5" s="1"/>
-      <c r="E5" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>329</v>
-      </c>
-      <c r="G5" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="I5" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="N5" s="1"/>
-      <c r="P5" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>69</v>
-      </c>
-      <c r="R5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="S5" t="s">
-        <v>106</v>
-      </c>
-      <c r="T5" t="s">
-        <v>88</v>
-      </c>
-      <c r="U5" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>107</v>
-      </c>
-      <c r="Z5" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB5" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="AC5" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AD5" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE5" t="s">
-        <v>109</v>
-      </c>
-      <c r="AF5" t="s">
-        <v>69</v>
-      </c>
-      <c r="AG5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH5" t="s">
-        <v>105</v>
-      </c>
-      <c r="AI5" t="s">
-        <v>69</v>
-      </c>
-      <c r="AJ5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK5" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL5" t="s">
-        <v>110</v>
-      </c>
-      <c r="AM5" t="s">
-        <v>111</v>
-      </c>
-      <c r="AN5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AO5" t="s">
-        <v>112</v>
-      </c>
-      <c r="AP5" t="s">
-        <v>113</v>
-      </c>
-      <c r="AQ5" t="s">
-        <v>114</v>
-      </c>
-      <c r="AR5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AU5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AV5" t="s">
-        <v>115</v>
-      </c>
+      <c r="R5" s="1"/>
+      <c r="AD5" s="1"/>
     </row>
     <row r="6" spans="1:50" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>116</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>117</v>
-      </c>
+      <c r="C6" s="1"/>
       <c r="D6" s="1"/>
-      <c r="E6" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="F6" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="G6" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="I6" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="K6" s="15">
-        <v>3713</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="M6" t="s">
-        <v>83</v>
-      </c>
-      <c r="N6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="P6" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>123</v>
-      </c>
-      <c r="R6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="S6" t="s">
-        <v>124</v>
-      </c>
-      <c r="T6" t="s">
-        <v>88</v>
-      </c>
-      <c r="U6" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>125</v>
-      </c>
-      <c r="Z6" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA6" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB6" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="AC6" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AD6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH6" t="s">
-        <v>122</v>
-      </c>
-      <c r="AI6" t="s">
-        <v>123</v>
-      </c>
-      <c r="AJ6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK6" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL6" t="s">
-        <v>127</v>
-      </c>
-      <c r="AM6" t="s">
-        <v>128</v>
-      </c>
-      <c r="AN6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AO6" t="s">
-        <v>129</v>
-      </c>
-      <c r="AP6" t="s">
-        <v>130</v>
-      </c>
-      <c r="AQ6" t="s">
-        <v>69</v>
-      </c>
-      <c r="AR6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AV6" t="s">
-        <v>131</v>
-      </c>
-      <c r="AW6" t="s">
-        <v>69</v>
-      </c>
-      <c r="AX6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:50" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <f t="shared" ref="A7:A12" si="1">ROW(B7) - 2</f>
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>132</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>133</v>
-      </c>
+      <c r="N6" s="1"/>
+      <c r="R6" s="1"/>
+      <c r="AD6" s="1"/>
+    </row>
+    <row r="7" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="C7" s="1"/>
       <c r="D7" s="1"/>
-      <c r="E7" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="G7" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="I7" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="K7" s="15">
-        <v>525</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="M7" t="s">
-        <v>83</v>
-      </c>
-      <c r="N7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="P7" t="s">
-        <v>135</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>86</v>
-      </c>
-      <c r="R7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="S7" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="T7" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="U7" s="14" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y7" s="15" t="s">
-        <v>137</v>
-      </c>
-      <c r="Z7" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="AA7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB7" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="AC7" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AD7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE7" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="AF7" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="AG7" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH7" t="s">
-        <v>135</v>
-      </c>
-      <c r="AI7" t="s">
-        <v>86</v>
-      </c>
-      <c r="AJ7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK7" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL7" t="s">
-        <v>93</v>
-      </c>
-      <c r="AM7" t="s">
-        <v>94</v>
-      </c>
-      <c r="AN7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AO7" t="s">
-        <v>95</v>
-      </c>
-      <c r="AP7" t="s">
-        <v>96</v>
-      </c>
-      <c r="AQ7" t="s">
-        <v>97</v>
-      </c>
-      <c r="AR7" t="b">
-        <v>1</v>
-      </c>
+      <c r="N7" s="1"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="15"/>
+      <c r="T7" s="15"/>
+      <c r="U7" s="14"/>
+      <c r="Y7" s="15"/>
+      <c r="Z7" s="15"/>
+      <c r="AE7" s="15"/>
+      <c r="AF7" s="15"/>
+      <c r="AG7" s="2"/>
     </row>
     <row r="8" spans="1:50" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>140</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>141</v>
-      </c>
+      <c r="C8" s="1"/>
       <c r="D8" s="1"/>
-      <c r="E8" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="G8" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H8" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="I8" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="J8" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="K8" s="15">
-        <v>5386</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="M8" t="s">
-        <v>83</v>
-      </c>
-      <c r="N8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O8" t="s">
-        <v>146</v>
-      </c>
-      <c r="P8" t="s">
-        <v>147</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>86</v>
-      </c>
-      <c r="R8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="S8" t="s">
-        <v>148</v>
-      </c>
-      <c r="T8" t="s">
-        <v>88</v>
-      </c>
-      <c r="U8" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y8" t="s">
-        <v>149</v>
-      </c>
-      <c r="Z8" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA8" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB8" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="AC8" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AD8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE8" t="s">
-        <v>151</v>
-      </c>
-      <c r="AF8" t="s">
-        <v>69</v>
-      </c>
-      <c r="AG8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH8" t="s">
-        <v>147</v>
-      </c>
-      <c r="AI8" t="s">
-        <v>86</v>
-      </c>
-      <c r="AJ8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK8" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL8" t="s">
-        <v>152</v>
-      </c>
-      <c r="AM8" t="s">
-        <v>153</v>
-      </c>
-      <c r="AN8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AO8" t="s">
-        <v>154</v>
-      </c>
-      <c r="AP8" t="s">
-        <v>155</v>
-      </c>
-      <c r="AQ8" t="s">
-        <v>69</v>
-      </c>
-      <c r="AR8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AV8" t="s">
-        <v>156</v>
-      </c>
-      <c r="AW8" t="s">
-        <v>69</v>
-      </c>
-      <c r="AX8" t="b">
-        <v>1</v>
-      </c>
+      <c r="J8" s="12"/>
+      <c r="N8" s="1"/>
+      <c r="R8" s="1"/>
+      <c r="AJ8" s="1"/>
+      <c r="AN8" s="1"/>
     </row>
     <row r="9" spans="1:50" ht="55.35" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <f t="shared" si="1"/>
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>157</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>158</v>
-      </c>
+      <c r="C9" s="1"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="G9" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="I9" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="K9" s="15">
-        <v>2735</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="M9" t="s">
-        <v>83</v>
-      </c>
-      <c r="N9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O9" t="s">
-        <v>163</v>
-      </c>
-      <c r="P9" t="s">
-        <v>164</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>165</v>
-      </c>
-      <c r="R9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="S9" t="s">
-        <v>166</v>
-      </c>
-      <c r="T9" t="s">
-        <v>88</v>
-      </c>
-      <c r="U9" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y9" t="s">
-        <v>167</v>
-      </c>
-      <c r="Z9" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB9" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="AC9" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AD9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH9" t="s">
-        <v>164</v>
-      </c>
-      <c r="AI9" t="s">
-        <v>169</v>
-      </c>
-      <c r="AJ9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK9" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL9" t="s">
-        <v>170</v>
-      </c>
-      <c r="AM9" t="s">
-        <v>171</v>
-      </c>
-      <c r="AN9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AO9" t="s">
-        <v>172</v>
-      </c>
-      <c r="AP9" t="s">
-        <v>173</v>
-      </c>
-      <c r="AQ9" t="s">
-        <v>97</v>
-      </c>
-      <c r="AR9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AV9" t="s">
-        <v>174</v>
-      </c>
-      <c r="AW9" t="s">
-        <v>69</v>
-      </c>
-      <c r="AX9" t="b">
-        <v>1</v>
-      </c>
+      <c r="N9" s="1"/>
+      <c r="R9" s="1"/>
+      <c r="AD9" s="1"/>
+      <c r="AN9" s="1"/>
     </row>
     <row r="10" spans="1:50" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <f t="shared" si="1"/>
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>175</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>176</v>
-      </c>
+      <c r="C10" s="1"/>
       <c r="D10" s="1"/>
-      <c r="E10" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>178</v>
-      </c>
-      <c r="G10" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="I10" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="M10" t="s">
-        <v>83</v>
-      </c>
-      <c r="N10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="P10" t="s">
-        <v>180</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>69</v>
-      </c>
-      <c r="R10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="S10" t="s">
-        <v>181</v>
-      </c>
-      <c r="T10" t="s">
-        <v>88</v>
-      </c>
-      <c r="U10" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y10" t="s">
-        <v>182</v>
-      </c>
-      <c r="Z10" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA10" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB10" t="s">
-        <v>183</v>
-      </c>
-      <c r="AC10" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="AD10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE10" t="s">
-        <v>184</v>
-      </c>
-      <c r="AF10" t="s">
-        <v>69</v>
-      </c>
-      <c r="AG10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH10" t="s">
-        <v>180</v>
-      </c>
-      <c r="AI10" t="s">
-        <v>69</v>
-      </c>
-      <c r="AJ10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK10" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL10" t="s">
-        <v>185</v>
-      </c>
-      <c r="AM10" t="s">
-        <v>186</v>
-      </c>
-      <c r="AN10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AO10" t="s">
-        <v>187</v>
-      </c>
-      <c r="AP10" t="s">
-        <v>313</v>
-      </c>
-      <c r="AQ10" t="s">
-        <v>314</v>
-      </c>
-      <c r="AR10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AV10" t="s">
-        <v>315</v>
-      </c>
-      <c r="AW10" t="s">
-        <v>69</v>
-      </c>
-      <c r="AX10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:50" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <f t="shared" si="1"/>
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>188</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>189</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>337</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="G11" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H11" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="I11" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="K11" s="15">
-        <v>6672</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="M11" t="s">
-        <v>83</v>
-      </c>
-      <c r="N11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O11" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="P11" s="12" t="s">
-        <v>190</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>192</v>
-      </c>
-      <c r="R11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="S11" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="T11" s="11" t="s">
-        <v>194</v>
-      </c>
-      <c r="U11" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="V11" s="11" t="s">
-        <v>195</v>
-      </c>
-      <c r="W11" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="X11" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y11" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="Z11" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="AA11" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB11" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="AC11" s="21" t="s">
-        <v>194</v>
-      </c>
-      <c r="AD11" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE11" s="12" t="s">
-        <v>198</v>
-      </c>
-      <c r="AF11" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="AG11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH11" t="s">
-        <v>190</v>
-      </c>
-      <c r="AI11" t="s">
-        <v>192</v>
-      </c>
-      <c r="AJ11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK11" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL11" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="AM11" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="AN11" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="AO11" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="AS11" t="s">
-        <v>75</v>
-      </c>
-      <c r="AT11" t="s">
-        <v>76</v>
-      </c>
-      <c r="AU11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AV11" t="s">
-        <v>199</v>
-      </c>
-      <c r="AW11" t="s">
-        <v>316</v>
-      </c>
-      <c r="AX11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:50" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="B12" t="s">
-        <v>200</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>201</v>
-      </c>
+      <c r="N10" s="1"/>
+      <c r="R10" s="1"/>
+      <c r="AB10"/>
+      <c r="AD10" s="1"/>
+      <c r="AN10" s="1"/>
+    </row>
+    <row r="11" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="12"/>
+      <c r="R11" s="1"/>
+      <c r="S11" s="2"/>
+      <c r="T11" s="11"/>
+      <c r="U11" s="11"/>
+      <c r="V11" s="11"/>
+      <c r="W11" s="11"/>
+      <c r="X11" s="11"/>
+      <c r="Y11" s="2"/>
+      <c r="Z11" s="12"/>
+      <c r="AA11" s="12"/>
+      <c r="AC11" s="21"/>
+      <c r="AD11" s="10"/>
+      <c r="AE11" s="12"/>
+      <c r="AF11" s="11"/>
+      <c r="AL11" s="11"/>
+      <c r="AM11" s="11"/>
+      <c r="AN11" s="11"/>
+      <c r="AO11" s="11"/>
+    </row>
+    <row r="12" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="C12" s="1"/>
       <c r="D12" s="1"/>
-      <c r="E12" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>202</v>
-      </c>
-      <c r="G12" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H12" s="12" t="s">
-        <v>203</v>
-      </c>
-      <c r="I12" s="12" t="s">
-        <v>203</v>
-      </c>
-      <c r="J12" s="12" t="s">
-        <v>203</v>
-      </c>
-      <c r="K12" s="15">
-        <v>7098</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="M12" t="s">
-        <v>83</v>
-      </c>
-      <c r="N12" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O12" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="P12" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>69</v>
-      </c>
-      <c r="R12" s="1" t="b">
-        <v>1</v>
-      </c>
+      <c r="J12" s="12"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="2"/>
+      <c r="P12" s="2"/>
+      <c r="R12" s="1"/>
       <c r="AD12" s="1"/>
       <c r="AN12" s="1"/>
     </row>
-    <row r="13" spans="1:50" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <f>ROW(B13) - 2</f>
-        <v>11</v>
-      </c>
-      <c r="B13" t="s">
-        <v>205</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>206</v>
-      </c>
+    <row r="13" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="C13" s="1"/>
       <c r="D13" s="1"/>
-      <c r="E13" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>208</v>
-      </c>
-      <c r="G13" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H13" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="I13" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="J13" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="M13" t="s">
-        <v>83</v>
-      </c>
-      <c r="N13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="O13" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="P13" t="s">
-        <v>210</v>
-      </c>
-      <c r="Q13" t="s">
-        <v>317</v>
-      </c>
-      <c r="R13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="S13" t="s">
-        <v>321</v>
-      </c>
-      <c r="T13" t="s">
-        <v>194</v>
-      </c>
-      <c r="U13" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y13" t="s">
-        <v>322</v>
-      </c>
-      <c r="Z13" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="AA13" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB13" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="AC13" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="AD13" s="10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH13" t="s">
-        <v>210</v>
-      </c>
-      <c r="AI13" t="s">
-        <v>317</v>
-      </c>
-      <c r="AJ13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK13" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL13" t="s">
-        <v>324</v>
-      </c>
-      <c r="AM13" t="s">
-        <v>171</v>
-      </c>
-      <c r="AN13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AO13" t="s">
-        <v>325</v>
-      </c>
-      <c r="AP13" t="s">
-        <v>326</v>
-      </c>
-      <c r="AQ13" t="s">
-        <v>327</v>
-      </c>
-      <c r="AR13" t="b">
-        <v>1</v>
-      </c>
-      <c r="AV13" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="AW13" t="s">
-        <v>69</v>
-      </c>
-      <c r="AX13" t="b">
-        <v>1</v>
-      </c>
+      <c r="J13" s="12"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="2"/>
+      <c r="R13" s="1"/>
+      <c r="AC13" s="12"/>
+      <c r="AD13" s="10"/>
+      <c r="AJ13" s="1"/>
+      <c r="AN13" s="1"/>
+      <c r="AV13" s="2"/>
     </row>
     <row r="14" spans="1:50" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <f>ROW(B14) - 2</f>
-        <v>12</v>
-      </c>
-      <c r="B14" t="s">
-        <v>212</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>213</v>
-      </c>
+      <c r="C14" s="1"/>
       <c r="D14" s="1"/>
-      <c r="E14" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>215</v>
-      </c>
-      <c r="G14" s="12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H14" s="12" t="s">
-        <v>216</v>
-      </c>
-      <c r="I14" s="12" t="s">
-        <v>216</v>
-      </c>
-      <c r="J14" s="12" t="s">
-        <v>216</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M14" t="s">
-        <v>218</v>
-      </c>
-      <c r="N14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="P14" t="s">
-        <v>217</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>218</v>
-      </c>
-      <c r="R14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="S14" t="s">
-        <v>219</v>
-      </c>
-      <c r="T14" t="s">
-        <v>88</v>
-      </c>
-      <c r="U14" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y14" t="s">
-        <v>220</v>
-      </c>
-      <c r="Z14" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA14" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB14" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="AC14" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AD14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AE14" t="s">
-        <v>222</v>
-      </c>
-      <c r="AF14" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="AG14" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH14" t="s">
-        <v>217</v>
-      </c>
-      <c r="AI14" t="s">
-        <v>218</v>
-      </c>
-      <c r="AJ14" t="b">
-        <v>1</v>
-      </c>
-      <c r="AK14" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL14" t="s">
-        <v>223</v>
-      </c>
-      <c r="AM14" t="s">
-        <v>224</v>
-      </c>
-      <c r="AN14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="AO14" t="s">
-        <v>225</v>
-      </c>
-      <c r="AP14" t="s">
-        <v>226</v>
-      </c>
-      <c r="AQ14" t="s">
-        <v>227</v>
-      </c>
-      <c r="AR14" t="b">
-        <v>1</v>
-      </c>
-      <c r="AV14" t="s">
-        <v>228</v>
-      </c>
-      <c r="AW14" t="s">
-        <v>115</v>
-      </c>
-      <c r="AX14" t="b">
-        <v>1</v>
-      </c>
+      <c r="J14" s="12"/>
+      <c r="N14" s="1"/>
+      <c r="R14" s="1"/>
+      <c r="AD14" s="1"/>
+      <c r="AF14" s="11"/>
+      <c r="AN14" s="1"/>
     </row>
     <row r="15" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <f>ROW(B15) - 2</f>
-        <v>13</v>
-      </c>
-      <c r="B15" t="s">
-        <v>330</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>331</v>
-      </c>
+      <c r="C15" s="1"/>
       <c r="D15" s="1"/>
-      <c r="E15" s="2" t="s">
-        <v>332</v>
-      </c>
-      <c r="F15" s="12" t="s">
-        <v>208</v>
-      </c>
-      <c r="G15" s="12" t="b">
-        <v>0</v>
-      </c>
-      <c r="H15" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="I15" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>209</v>
-      </c>
       <c r="N15" s="1"/>
       <c r="R15" s="1"/>
       <c r="AD15" s="1"/>
       <c r="AN15" s="1"/>
     </row>
-    <row r="16" spans="1:50" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <f>ROW(B16) - 2</f>
-        <v>14</v>
-      </c>
-      <c r="B16" t="s">
-        <v>333</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>334</v>
-      </c>
+    <row r="16" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="C16" s="1"/>
       <c r="D16" s="1"/>
-      <c r="E16" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="G16" s="12" t="b">
-        <v>0</v>
-      </c>
       <c r="N16" s="1"/>
       <c r="R16" s="1"/>
       <c r="AD16" s="1"/>
@@ -3781,12 +2083,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="AH1:AX1"/>
     <mergeCell ref="E1:N1"/>
     <mergeCell ref="S1:AD1"/>
     <mergeCell ref="P1:R1"/>
     <mergeCell ref="AE1:AG1"/>
-    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <hyperlinks>
@@ -3853,13 +2155,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>229</v>
+        <v>75</v>
       </c>
       <c r="B1" t="s">
-        <v>230</v>
+        <v>76</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>231</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -3867,10 +2169,10 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>232</v>
+        <v>78</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>233</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -3878,10 +2180,10 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>234</v>
+        <v>80</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>235</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -3889,10 +2191,10 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>236</v>
+        <v>82</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>237</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -3900,10 +2202,10 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>238</v>
+        <v>84</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>239</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -3911,10 +2213,10 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>240</v>
+        <v>86</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>241</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -3922,10 +2224,10 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>242</v>
+        <v>88</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>243</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -3933,10 +2235,10 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>244</v>
+        <v>90</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>245</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -3944,10 +2246,10 @@
         <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>246</v>
+        <v>92</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>247</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -3955,21 +2257,21 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>248</v>
+        <v>94</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>250</v>
+        <v>96</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>251</v>
+        <v>173</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -3977,10 +2279,10 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>252</v>
+        <v>97</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>253</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -3988,10 +2290,10 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>254</v>
+        <v>99</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>255</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -3999,10 +2301,10 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>256</v>
+        <v>101</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>243</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4010,10 +2312,10 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>257</v>
+        <v>102</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>258</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
@@ -4021,10 +2323,10 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>259</v>
+        <v>104</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>260</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4032,10 +2334,10 @@
         <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>261</v>
+        <v>106</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>262</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4043,10 +2345,10 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>263</v>
+        <v>108</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>243</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4054,10 +2356,10 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>264</v>
+        <v>109</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>265</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4065,10 +2367,10 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>266</v>
+        <v>111</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>267</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4076,10 +2378,10 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>268</v>
+        <v>113</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>243</v>
+        <v>89</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4087,10 +2389,10 @@
         <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>269</v>
+        <v>114</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>270</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4098,10 +2400,10 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>271</v>
+        <v>116</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>272</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4109,10 +2411,10 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>273</v>
+        <v>118</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>243</v>
+        <v>89</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4120,10 +2422,10 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>274</v>
+        <v>119</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>275</v>
+        <v>120</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4131,10 +2433,10 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>276</v>
+        <v>121</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>277</v>
+        <v>122</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4142,10 +2444,10 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>278</v>
+        <v>123</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>243</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4153,10 +2455,10 @@
         <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>279</v>
+        <v>124</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>280</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4164,10 +2466,10 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>281</v>
+        <v>126</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>282</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4175,10 +2477,10 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>283</v>
+        <v>128</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>243</v>
+        <v>89</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4186,10 +2488,10 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>284</v>
+        <v>129</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>285</v>
+        <v>130</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4197,10 +2499,10 @@
         <v>36</v>
       </c>
       <c r="B32" t="s">
-        <v>286</v>
+        <v>131</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>287</v>
+        <v>132</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4208,10 +2510,10 @@
         <v>37</v>
       </c>
       <c r="B33" t="s">
-        <v>288</v>
+        <v>133</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>243</v>
+        <v>89</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4219,10 +2521,10 @@
         <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>289</v>
+        <v>134</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>290</v>
+        <v>135</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4230,10 +2532,10 @@
         <v>39</v>
       </c>
       <c r="B35" t="s">
-        <v>291</v>
+        <v>136</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>292</v>
+        <v>137</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4241,10 +2543,10 @@
         <v>40</v>
       </c>
       <c r="B36" t="s">
-        <v>293</v>
+        <v>138</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>243</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4252,10 +2554,10 @@
         <v>41</v>
       </c>
       <c r="B37" t="s">
-        <v>294</v>
+        <v>139</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>295</v>
+        <v>140</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4263,10 +2565,10 @@
         <v>42</v>
       </c>
       <c r="B38" t="s">
-        <v>296</v>
+        <v>141</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>297</v>
+        <v>142</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4274,10 +2576,10 @@
         <v>43</v>
       </c>
       <c r="B39" t="s">
-        <v>298</v>
+        <v>143</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>299</v>
+        <v>144</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4285,10 +2587,10 @@
         <v>44</v>
       </c>
       <c r="B40" t="s">
-        <v>300</v>
+        <v>145</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>243</v>
+        <v>89</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
@@ -4296,10 +2598,10 @@
         <v>45</v>
       </c>
       <c r="B41" t="s">
-        <v>301</v>
+        <v>146</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>302</v>
+        <v>147</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4307,10 +2609,10 @@
         <v>46</v>
       </c>
       <c r="B42" t="s">
-        <v>303</v>
+        <v>148</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>304</v>
+        <v>149</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4318,10 +2620,10 @@
         <v>47</v>
       </c>
       <c r="B43" t="s">
-        <v>305</v>
+        <v>150</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>306</v>
+        <v>151</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4329,10 +2631,10 @@
         <v>48</v>
       </c>
       <c r="B44" t="s">
-        <v>307</v>
+        <v>152</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>243</v>
+        <v>89</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4340,10 +2642,10 @@
         <v>49</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>308</v>
+        <v>153</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>309</v>
+        <v>154</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
@@ -4351,10 +2653,10 @@
         <v>50</v>
       </c>
       <c r="B46" t="s">
-        <v>310</v>
+        <v>155</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>311</v>
+        <v>156</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
@@ -4362,10 +2664,10 @@
         <v>51</v>
       </c>
       <c r="B47" t="s">
-        <v>312</v>
+        <v>157</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>243</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>